<commit_message>
Update Nội dung công việc hàng ngày.xlsx
</commit_message>
<xml_diff>
--- a/5. Other/Nội dung công việc hàng ngày.xlsx
+++ b/5. Other/Nội dung công việc hàng ngày.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\VNET\5. Other\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2AD61C0B-D9FA-4763-A573-1C71E8E39436}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91D80F23-1BC1-40C0-A778-9EC9F06B1BBF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="3" xr2:uid="{F20CEA29-D7AE-4CD4-9104-84E191A61AC3}"/>
   </bookViews>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="325" uniqueCount="173">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="329" uniqueCount="173">
   <si>
     <t>Hoàn thiện 73 dây nguồn VNSH03</t>
   </si>
@@ -926,6 +926,30 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="17" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -941,80 +965,56 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="17" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="17" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="17" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -1344,15 +1344,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A1" s="62">
+      <c r="A1" s="70">
         <v>46174</v>
       </c>
-      <c r="B1" s="63"/>
-      <c r="C1" s="63"/>
-      <c r="D1" s="63"/>
-      <c r="E1" s="63"/>
-      <c r="F1" s="63"/>
-      <c r="G1" s="63"/>
+      <c r="B1" s="71"/>
+      <c r="C1" s="71"/>
+      <c r="D1" s="71"/>
+      <c r="E1" s="71"/>
+      <c r="F1" s="71"/>
+      <c r="G1" s="71"/>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
@@ -1361,146 +1361,146 @@
       <c r="B2" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C2" s="64" t="s">
+      <c r="C2" s="72" t="s">
         <v>8</v>
       </c>
-      <c r="D2" s="65"/>
-      <c r="E2" s="65"/>
-      <c r="F2" s="65"/>
-      <c r="G2" s="66"/>
+      <c r="D2" s="73"/>
+      <c r="E2" s="73"/>
+      <c r="F2" s="73"/>
+      <c r="G2" s="74"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3" s="71">
+      <c r="A3" s="65">
         <v>46202</v>
       </c>
-      <c r="B3" s="67" t="s">
+      <c r="B3" s="66" t="s">
         <v>5</v>
       </c>
-      <c r="C3" s="67" t="s">
+      <c r="C3" s="66" t="s">
         <v>2</v>
       </c>
-      <c r="D3" s="67"/>
-      <c r="E3" s="67"/>
-      <c r="F3" s="67"/>
-      <c r="G3" s="67"/>
+      <c r="D3" s="66"/>
+      <c r="E3" s="66"/>
+      <c r="F3" s="66"/>
+      <c r="G3" s="66"/>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4" s="71"/>
-      <c r="B4" s="67"/>
-      <c r="C4" s="67" t="s">
+      <c r="A4" s="65"/>
+      <c r="B4" s="66"/>
+      <c r="C4" s="66" t="s">
         <v>0</v>
       </c>
-      <c r="D4" s="67"/>
-      <c r="E4" s="67"/>
-      <c r="F4" s="67"/>
-      <c r="G4" s="67"/>
+      <c r="D4" s="66"/>
+      <c r="E4" s="66"/>
+      <c r="F4" s="66"/>
+      <c r="G4" s="66"/>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" s="71"/>
-      <c r="B5" s="67"/>
-      <c r="C5" s="67" t="s">
+      <c r="A5" s="65"/>
+      <c r="B5" s="66"/>
+      <c r="C5" s="66" t="s">
         <v>3</v>
       </c>
-      <c r="D5" s="67"/>
-      <c r="E5" s="67"/>
-      <c r="F5" s="67"/>
-      <c r="G5" s="67"/>
+      <c r="D5" s="66"/>
+      <c r="E5" s="66"/>
+      <c r="F5" s="66"/>
+      <c r="G5" s="66"/>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" s="71"/>
-      <c r="B6" s="67" t="s">
-        <v>4</v>
-      </c>
-      <c r="C6" s="67" t="s">
+      <c r="A6" s="65"/>
+      <c r="B6" s="66" t="s">
+        <v>4</v>
+      </c>
+      <c r="C6" s="66" t="s">
         <v>1</v>
       </c>
-      <c r="D6" s="67"/>
-      <c r="E6" s="67"/>
-      <c r="F6" s="67"/>
-      <c r="G6" s="67"/>
+      <c r="D6" s="66"/>
+      <c r="E6" s="66"/>
+      <c r="F6" s="66"/>
+      <c r="G6" s="66"/>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A7" s="71"/>
-      <c r="B7" s="67"/>
-      <c r="C7" s="67" t="s">
+      <c r="A7" s="65"/>
+      <c r="B7" s="66"/>
+      <c r="C7" s="66" t="s">
         <v>10</v>
       </c>
-      <c r="D7" s="67"/>
-      <c r="E7" s="67"/>
-      <c r="F7" s="67"/>
-      <c r="G7" s="67"/>
+      <c r="D7" s="66"/>
+      <c r="E7" s="66"/>
+      <c r="F7" s="66"/>
+      <c r="G7" s="66"/>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A8" s="71"/>
-      <c r="B8" s="67"/>
-      <c r="C8" s="67" t="s">
+      <c r="A8" s="65"/>
+      <c r="B8" s="66"/>
+      <c r="C8" s="66" t="s">
         <v>9</v>
       </c>
-      <c r="D8" s="67"/>
-      <c r="E8" s="67"/>
-      <c r="F8" s="67"/>
-      <c r="G8" s="67"/>
+      <c r="D8" s="66"/>
+      <c r="E8" s="66"/>
+      <c r="F8" s="66"/>
+      <c r="G8" s="66"/>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A9" s="71">
+      <c r="A9" s="65">
         <v>46203</v>
       </c>
-      <c r="B9" s="67" t="s">
+      <c r="B9" s="66" t="s">
         <v>5</v>
       </c>
-      <c r="C9" s="72" t="s">
+      <c r="C9" s="67" t="s">
         <v>11</v>
       </c>
-      <c r="D9" s="73"/>
-      <c r="E9" s="73"/>
-      <c r="F9" s="73"/>
-      <c r="G9" s="74"/>
+      <c r="D9" s="68"/>
+      <c r="E9" s="68"/>
+      <c r="F9" s="68"/>
+      <c r="G9" s="69"/>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A10" s="71"/>
-      <c r="B10" s="67"/>
-      <c r="C10" s="68" t="s">
+      <c r="A10" s="65"/>
+      <c r="B10" s="66"/>
+      <c r="C10" s="62" t="s">
         <v>12</v>
       </c>
-      <c r="D10" s="69"/>
-      <c r="E10" s="69"/>
-      <c r="F10" s="69"/>
-      <c r="G10" s="70"/>
+      <c r="D10" s="63"/>
+      <c r="E10" s="63"/>
+      <c r="F10" s="63"/>
+      <c r="G10" s="64"/>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A11" s="71"/>
-      <c r="B11" s="67"/>
-      <c r="C11" s="68" t="s">
+      <c r="A11" s="65"/>
+      <c r="B11" s="66"/>
+      <c r="C11" s="62" t="s">
         <v>13</v>
       </c>
-      <c r="D11" s="69"/>
-      <c r="E11" s="69"/>
-      <c r="F11" s="69"/>
-      <c r="G11" s="70"/>
+      <c r="D11" s="63"/>
+      <c r="E11" s="63"/>
+      <c r="F11" s="63"/>
+      <c r="G11" s="64"/>
     </row>
     <row r="12" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="71"/>
-      <c r="B12" s="67"/>
-      <c r="C12" s="68" t="s">
+      <c r="A12" s="65"/>
+      <c r="B12" s="66"/>
+      <c r="C12" s="62" t="s">
         <v>14</v>
       </c>
-      <c r="D12" s="69"/>
-      <c r="E12" s="69"/>
-      <c r="F12" s="69"/>
-      <c r="G12" s="70"/>
+      <c r="D12" s="63"/>
+      <c r="E12" s="63"/>
+      <c r="F12" s="63"/>
+      <c r="G12" s="64"/>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A13" s="71"/>
+      <c r="A13" s="65"/>
       <c r="B13" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="C13" s="68" t="s">
+      <c r="C13" s="62" t="s">
         <v>9</v>
       </c>
-      <c r="D13" s="69"/>
-      <c r="E13" s="69"/>
-      <c r="F13" s="69"/>
-      <c r="G13" s="70"/>
+      <c r="D13" s="63"/>
+      <c r="E13" s="63"/>
+      <c r="F13" s="63"/>
+      <c r="G13" s="64"/>
     </row>
   </sheetData>
   <autoFilter ref="A2:G8" xr:uid="{5B424F82-FB95-405B-80D1-35D47957B3B0}">
@@ -1510,14 +1510,6 @@
     <filterColumn colId="5" showButton="0"/>
   </autoFilter>
   <mergeCells count="18">
-    <mergeCell ref="C12:G12"/>
-    <mergeCell ref="C13:G13"/>
-    <mergeCell ref="A9:A13"/>
-    <mergeCell ref="B9:B12"/>
-    <mergeCell ref="A3:A8"/>
-    <mergeCell ref="C9:G9"/>
-    <mergeCell ref="C10:G10"/>
-    <mergeCell ref="C11:G11"/>
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="C2:G2"/>
     <mergeCell ref="B6:B8"/>
@@ -1528,6 +1520,14 @@
     <mergeCell ref="C5:G5"/>
     <mergeCell ref="C6:G6"/>
     <mergeCell ref="C7:G7"/>
+    <mergeCell ref="C12:G12"/>
+    <mergeCell ref="C13:G13"/>
+    <mergeCell ref="A9:A13"/>
+    <mergeCell ref="B9:B12"/>
+    <mergeCell ref="A3:A8"/>
+    <mergeCell ref="C9:G9"/>
+    <mergeCell ref="C10:G10"/>
+    <mergeCell ref="C11:G11"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1545,15 +1545,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A1" s="87">
+      <c r="A1" s="78">
         <v>46204</v>
       </c>
-      <c r="B1" s="87"/>
-      <c r="C1" s="87"/>
-      <c r="D1" s="87"/>
-      <c r="E1" s="87"/>
-      <c r="F1" s="87"/>
-      <c r="G1" s="87"/>
+      <c r="B1" s="78"/>
+      <c r="C1" s="78"/>
+      <c r="D1" s="78"/>
+      <c r="E1" s="78"/>
+      <c r="F1" s="78"/>
+      <c r="G1" s="78"/>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
@@ -1562,152 +1562,152 @@
       <c r="B2" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C2" s="88" t="s">
+      <c r="C2" s="79" t="s">
         <v>8</v>
       </c>
-      <c r="D2" s="88"/>
-      <c r="E2" s="88"/>
-      <c r="F2" s="88"/>
-      <c r="G2" s="88"/>
+      <c r="D2" s="79"/>
+      <c r="E2" s="79"/>
+      <c r="F2" s="79"/>
+      <c r="G2" s="79"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3" s="71">
+      <c r="A3" s="65">
         <v>46204</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="C3" s="67" t="s">
+      <c r="C3" s="66" t="s">
         <v>15</v>
       </c>
-      <c r="D3" s="67"/>
-      <c r="E3" s="67"/>
-      <c r="F3" s="67"/>
-      <c r="G3" s="67"/>
+      <c r="D3" s="66"/>
+      <c r="E3" s="66"/>
+      <c r="F3" s="66"/>
+      <c r="G3" s="66"/>
     </row>
     <row r="4" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="71"/>
-      <c r="B4" s="67" t="s">
-        <v>4</v>
-      </c>
-      <c r="C4" s="76" t="s">
+      <c r="A4" s="65"/>
+      <c r="B4" s="66" t="s">
+        <v>4</v>
+      </c>
+      <c r="C4" s="80" t="s">
         <v>16</v>
       </c>
-      <c r="D4" s="76"/>
-      <c r="E4" s="76"/>
-      <c r="F4" s="76"/>
-      <c r="G4" s="76"/>
+      <c r="D4" s="80"/>
+      <c r="E4" s="80"/>
+      <c r="F4" s="80"/>
+      <c r="G4" s="80"/>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" s="71"/>
-      <c r="B5" s="67"/>
-      <c r="C5" s="67" t="s">
+      <c r="A5" s="65"/>
+      <c r="B5" s="66"/>
+      <c r="C5" s="66" t="s">
         <v>17</v>
       </c>
-      <c r="D5" s="67"/>
-      <c r="E5" s="67"/>
-      <c r="F5" s="67"/>
-      <c r="G5" s="67"/>
+      <c r="D5" s="66"/>
+      <c r="E5" s="66"/>
+      <c r="F5" s="66"/>
+      <c r="G5" s="66"/>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" s="71"/>
-      <c r="B6" s="67"/>
-      <c r="C6" s="67" t="s">
+      <c r="A6" s="65"/>
+      <c r="B6" s="66"/>
+      <c r="C6" s="66" t="s">
         <v>18</v>
       </c>
-      <c r="D6" s="67"/>
-      <c r="E6" s="67"/>
-      <c r="F6" s="67"/>
-      <c r="G6" s="67"/>
+      <c r="D6" s="66"/>
+      <c r="E6" s="66"/>
+      <c r="F6" s="66"/>
+      <c r="G6" s="66"/>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A7" s="89">
+      <c r="A7" s="81">
         <v>46205</v>
       </c>
-      <c r="B7" s="78" t="s">
+      <c r="B7" s="75" t="s">
         <v>5</v>
       </c>
-      <c r="C7" s="72" t="s">
+      <c r="C7" s="67" t="s">
         <v>25</v>
       </c>
-      <c r="D7" s="73"/>
-      <c r="E7" s="73"/>
-      <c r="F7" s="73"/>
-      <c r="G7" s="74"/>
+      <c r="D7" s="68"/>
+      <c r="E7" s="68"/>
+      <c r="F7" s="68"/>
+      <c r="G7" s="69"/>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A8" s="90"/>
-      <c r="B8" s="86"/>
-      <c r="C8" s="68" t="s">
+      <c r="A8" s="82"/>
+      <c r="B8" s="77"/>
+      <c r="C8" s="62" t="s">
         <v>19</v>
       </c>
-      <c r="D8" s="69"/>
-      <c r="E8" s="69"/>
-      <c r="F8" s="69"/>
-      <c r="G8" s="70"/>
+      <c r="D8" s="63"/>
+      <c r="E8" s="63"/>
+      <c r="F8" s="63"/>
+      <c r="G8" s="64"/>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A9" s="90"/>
-      <c r="B9" s="79"/>
-      <c r="C9" s="68" t="s">
+      <c r="A9" s="82"/>
+      <c r="B9" s="76"/>
+      <c r="C9" s="62" t="s">
         <v>24</v>
       </c>
-      <c r="D9" s="69"/>
-      <c r="E9" s="69"/>
-      <c r="F9" s="69"/>
-      <c r="G9" s="70"/>
+      <c r="D9" s="63"/>
+      <c r="E9" s="63"/>
+      <c r="F9" s="63"/>
+      <c r="G9" s="64"/>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A10" s="90"/>
-      <c r="B10" s="67" t="s">
-        <v>4</v>
-      </c>
-      <c r="C10" s="68" t="s">
+      <c r="A10" s="82"/>
+      <c r="B10" s="66" t="s">
+        <v>4</v>
+      </c>
+      <c r="C10" s="62" t="s">
         <v>22</v>
       </c>
-      <c r="D10" s="69"/>
-      <c r="E10" s="69"/>
-      <c r="F10" s="69"/>
-      <c r="G10" s="70"/>
+      <c r="D10" s="63"/>
+      <c r="E10" s="63"/>
+      <c r="F10" s="63"/>
+      <c r="G10" s="64"/>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A11" s="90"/>
-      <c r="B11" s="67"/>
-      <c r="C11" s="68" t="s">
+      <c r="A11" s="82"/>
+      <c r="B11" s="66"/>
+      <c r="C11" s="62" t="s">
         <v>20</v>
       </c>
-      <c r="D11" s="69"/>
-      <c r="E11" s="69"/>
-      <c r="F11" s="69"/>
-      <c r="G11" s="70"/>
+      <c r="D11" s="63"/>
+      <c r="E11" s="63"/>
+      <c r="F11" s="63"/>
+      <c r="G11" s="64"/>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A12" s="90"/>
-      <c r="B12" s="67"/>
-      <c r="C12" s="68" t="s">
+      <c r="A12" s="82"/>
+      <c r="B12" s="66"/>
+      <c r="C12" s="62" t="s">
         <v>21</v>
       </c>
-      <c r="D12" s="69"/>
-      <c r="E12" s="69"/>
-      <c r="F12" s="69"/>
-      <c r="G12" s="70"/>
+      <c r="D12" s="63"/>
+      <c r="E12" s="63"/>
+      <c r="F12" s="63"/>
+      <c r="G12" s="64"/>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A13" s="91"/>
-      <c r="B13" s="67"/>
-      <c r="C13" s="68" t="s">
+      <c r="A13" s="83"/>
+      <c r="B13" s="66"/>
+      <c r="C13" s="62" t="s">
         <v>23</v>
       </c>
-      <c r="D13" s="69"/>
-      <c r="E13" s="69"/>
-      <c r="F13" s="69"/>
-      <c r="G13" s="70"/>
+      <c r="D13" s="63"/>
+      <c r="E13" s="63"/>
+      <c r="F13" s="63"/>
+      <c r="G13" s="64"/>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A14" s="80">
+      <c r="A14" s="85">
         <v>46206</v>
       </c>
-      <c r="B14" s="78" t="s">
+      <c r="B14" s="75" t="s">
         <v>5</v>
       </c>
       <c r="C14" s="3" t="s">
@@ -1719,348 +1719,348 @@
       <c r="G14" s="5"/>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A15" s="83"/>
-      <c r="B15" s="86"/>
-      <c r="C15" s="72" t="s">
+      <c r="A15" s="86"/>
+      <c r="B15" s="77"/>
+      <c r="C15" s="67" t="s">
         <v>26</v>
       </c>
-      <c r="D15" s="73"/>
-      <c r="E15" s="73"/>
-      <c r="F15" s="73"/>
-      <c r="G15" s="74"/>
+      <c r="D15" s="68"/>
+      <c r="E15" s="68"/>
+      <c r="F15" s="68"/>
+      <c r="G15" s="69"/>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A16" s="83"/>
-      <c r="B16" s="86"/>
-      <c r="C16" s="72" t="s">
+      <c r="A16" s="86"/>
+      <c r="B16" s="77"/>
+      <c r="C16" s="67" t="s">
         <v>28</v>
       </c>
-      <c r="D16" s="73"/>
-      <c r="E16" s="73"/>
-      <c r="F16" s="73"/>
-      <c r="G16" s="74"/>
+      <c r="D16" s="68"/>
+      <c r="E16" s="68"/>
+      <c r="F16" s="68"/>
+      <c r="G16" s="69"/>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A17" s="83"/>
-      <c r="B17" s="79"/>
-      <c r="C17" s="72" t="s">
+      <c r="A17" s="86"/>
+      <c r="B17" s="76"/>
+      <c r="C17" s="67" t="s">
         <v>27</v>
       </c>
-      <c r="D17" s="73"/>
-      <c r="E17" s="73"/>
-      <c r="F17" s="73"/>
-      <c r="G17" s="74"/>
+      <c r="D17" s="68"/>
+      <c r="E17" s="68"/>
+      <c r="F17" s="68"/>
+      <c r="G17" s="69"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A18" s="83"/>
-      <c r="B18" s="78" t="s">
-        <v>4</v>
-      </c>
-      <c r="C18" s="72" t="s">
+      <c r="A18" s="86"/>
+      <c r="B18" s="75" t="s">
+        <v>4</v>
+      </c>
+      <c r="C18" s="67" t="s">
         <v>29</v>
       </c>
-      <c r="D18" s="73"/>
-      <c r="E18" s="73"/>
-      <c r="F18" s="73"/>
-      <c r="G18" s="74"/>
+      <c r="D18" s="68"/>
+      <c r="E18" s="68"/>
+      <c r="F18" s="68"/>
+      <c r="G18" s="69"/>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A19" s="81"/>
-      <c r="B19" s="79"/>
-      <c r="C19" s="72" t="s">
+      <c r="A19" s="87"/>
+      <c r="B19" s="76"/>
+      <c r="C19" s="67" t="s">
         <v>31</v>
       </c>
-      <c r="D19" s="73"/>
-      <c r="E19" s="73"/>
-      <c r="F19" s="73"/>
-      <c r="G19" s="74"/>
+      <c r="D19" s="68"/>
+      <c r="E19" s="68"/>
+      <c r="F19" s="68"/>
+      <c r="G19" s="69"/>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A20" s="84">
+      <c r="A20" s="88">
         <v>46209</v>
       </c>
-      <c r="B20" s="67" t="s">
+      <c r="B20" s="66" t="s">
         <v>5</v>
       </c>
-      <c r="C20" s="67" t="s">
+      <c r="C20" s="66" t="s">
         <v>33</v>
       </c>
-      <c r="D20" s="67"/>
-      <c r="E20" s="67"/>
-      <c r="F20" s="67"/>
-      <c r="G20" s="67"/>
+      <c r="D20" s="66"/>
+      <c r="E20" s="66"/>
+      <c r="F20" s="66"/>
+      <c r="G20" s="66"/>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A21" s="84"/>
-      <c r="B21" s="67"/>
-      <c r="C21" s="67" t="s">
+      <c r="A21" s="88"/>
+      <c r="B21" s="66"/>
+      <c r="C21" s="66" t="s">
         <v>34</v>
       </c>
-      <c r="D21" s="67"/>
-      <c r="E21" s="67"/>
-      <c r="F21" s="67"/>
-      <c r="G21" s="67"/>
+      <c r="D21" s="66"/>
+      <c r="E21" s="66"/>
+      <c r="F21" s="66"/>
+      <c r="G21" s="66"/>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A22" s="84"/>
-      <c r="B22" s="67"/>
-      <c r="C22" s="67" t="s">
+      <c r="A22" s="88"/>
+      <c r="B22" s="66"/>
+      <c r="C22" s="66" t="s">
         <v>15</v>
       </c>
-      <c r="D22" s="67"/>
-      <c r="E22" s="67"/>
-      <c r="F22" s="67"/>
-      <c r="G22" s="67"/>
+      <c r="D22" s="66"/>
+      <c r="E22" s="66"/>
+      <c r="F22" s="66"/>
+      <c r="G22" s="66"/>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A23" s="84"/>
-      <c r="B23" s="67" t="s">
-        <v>4</v>
-      </c>
-      <c r="C23" s="67" t="s">
+      <c r="A23" s="88"/>
+      <c r="B23" s="66" t="s">
+        <v>4</v>
+      </c>
+      <c r="C23" s="66" t="s">
         <v>32</v>
       </c>
-      <c r="D23" s="67"/>
-      <c r="E23" s="67"/>
-      <c r="F23" s="67"/>
-      <c r="G23" s="67"/>
+      <c r="D23" s="66"/>
+      <c r="E23" s="66"/>
+      <c r="F23" s="66"/>
+      <c r="G23" s="66"/>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A24" s="84"/>
-      <c r="B24" s="67"/>
-      <c r="C24" s="72" t="s">
+      <c r="A24" s="88"/>
+      <c r="B24" s="66"/>
+      <c r="C24" s="67" t="s">
         <v>35</v>
       </c>
-      <c r="D24" s="73"/>
-      <c r="E24" s="73"/>
-      <c r="F24" s="73"/>
-      <c r="G24" s="74"/>
+      <c r="D24" s="68"/>
+      <c r="E24" s="68"/>
+      <c r="F24" s="68"/>
+      <c r="G24" s="69"/>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A25" s="84"/>
-      <c r="B25" s="67"/>
-      <c r="C25" s="72" t="s">
+      <c r="A25" s="88"/>
+      <c r="B25" s="66"/>
+      <c r="C25" s="67" t="s">
         <v>36</v>
       </c>
-      <c r="D25" s="73"/>
-      <c r="E25" s="73"/>
-      <c r="F25" s="73"/>
-      <c r="G25" s="74"/>
+      <c r="D25" s="68"/>
+      <c r="E25" s="68"/>
+      <c r="F25" s="68"/>
+      <c r="G25" s="69"/>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A26" s="84"/>
-      <c r="B26" s="67"/>
-      <c r="C26" s="72" t="s">
+      <c r="A26" s="88"/>
+      <c r="B26" s="66"/>
+      <c r="C26" s="67" t="s">
         <v>37</v>
       </c>
-      <c r="D26" s="73"/>
-      <c r="E26" s="73"/>
-      <c r="F26" s="73"/>
-      <c r="G26" s="74"/>
+      <c r="D26" s="68"/>
+      <c r="E26" s="68"/>
+      <c r="F26" s="68"/>
+      <c r="G26" s="69"/>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A27" s="84"/>
-      <c r="B27" s="67"/>
-      <c r="C27" s="72" t="s">
+      <c r="A27" s="88"/>
+      <c r="B27" s="66"/>
+      <c r="C27" s="67" t="s">
         <v>38</v>
       </c>
-      <c r="D27" s="73"/>
-      <c r="E27" s="73"/>
-      <c r="F27" s="73"/>
-      <c r="G27" s="74"/>
+      <c r="D27" s="68"/>
+      <c r="E27" s="68"/>
+      <c r="F27" s="68"/>
+      <c r="G27" s="69"/>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A28" s="84"/>
-      <c r="B28" s="67"/>
-      <c r="C28" s="72" t="s">
+      <c r="A28" s="88"/>
+      <c r="B28" s="66"/>
+      <c r="C28" s="67" t="s">
         <v>39</v>
       </c>
-      <c r="D28" s="73"/>
-      <c r="E28" s="73"/>
-      <c r="F28" s="73"/>
-      <c r="G28" s="74"/>
+      <c r="D28" s="68"/>
+      <c r="E28" s="68"/>
+      <c r="F28" s="68"/>
+      <c r="G28" s="69"/>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A29" s="84"/>
-      <c r="B29" s="67"/>
-      <c r="C29" s="72" t="s">
+      <c r="A29" s="88"/>
+      <c r="B29" s="66"/>
+      <c r="C29" s="67" t="s">
         <v>40</v>
       </c>
-      <c r="D29" s="73"/>
-      <c r="E29" s="73"/>
-      <c r="F29" s="73"/>
-      <c r="G29" s="74"/>
+      <c r="D29" s="68"/>
+      <c r="E29" s="68"/>
+      <c r="F29" s="68"/>
+      <c r="G29" s="69"/>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A30" s="84"/>
-      <c r="B30" s="67"/>
-      <c r="C30" s="72" t="s">
+      <c r="A30" s="88"/>
+      <c r="B30" s="66"/>
+      <c r="C30" s="67" t="s">
         <v>45</v>
       </c>
-      <c r="D30" s="73"/>
-      <c r="E30" s="73"/>
-      <c r="F30" s="73"/>
-      <c r="G30" s="74"/>
+      <c r="D30" s="68"/>
+      <c r="E30" s="68"/>
+      <c r="F30" s="68"/>
+      <c r="G30" s="69"/>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A31" s="84"/>
-      <c r="B31" s="67"/>
-      <c r="C31" s="72" t="s">
+      <c r="A31" s="88"/>
+      <c r="B31" s="66"/>
+      <c r="C31" s="67" t="s">
         <v>41</v>
       </c>
-      <c r="D31" s="73"/>
-      <c r="E31" s="73"/>
-      <c r="F31" s="73"/>
-      <c r="G31" s="74"/>
+      <c r="D31" s="68"/>
+      <c r="E31" s="68"/>
+      <c r="F31" s="68"/>
+      <c r="G31" s="69"/>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A32" s="84"/>
-      <c r="B32" s="67"/>
-      <c r="C32" s="72" t="s">
+      <c r="A32" s="88"/>
+      <c r="B32" s="66"/>
+      <c r="C32" s="67" t="s">
         <v>42</v>
       </c>
-      <c r="D32" s="73"/>
-      <c r="E32" s="73"/>
-      <c r="F32" s="73"/>
-      <c r="G32" s="74"/>
+      <c r="D32" s="68"/>
+      <c r="E32" s="68"/>
+      <c r="F32" s="68"/>
+      <c r="G32" s="69"/>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A33" s="84"/>
-      <c r="B33" s="67"/>
-      <c r="C33" s="72" t="s">
+      <c r="A33" s="88"/>
+      <c r="B33" s="66"/>
+      <c r="C33" s="67" t="s">
         <v>43</v>
       </c>
-      <c r="D33" s="73"/>
-      <c r="E33" s="73"/>
-      <c r="F33" s="73"/>
-      <c r="G33" s="74"/>
+      <c r="D33" s="68"/>
+      <c r="E33" s="68"/>
+      <c r="F33" s="68"/>
+      <c r="G33" s="69"/>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A34" s="84"/>
-      <c r="B34" s="67"/>
-      <c r="C34" s="72" t="s">
+      <c r="A34" s="88"/>
+      <c r="B34" s="66"/>
+      <c r="C34" s="67" t="s">
         <v>44</v>
       </c>
-      <c r="D34" s="73"/>
-      <c r="E34" s="73"/>
-      <c r="F34" s="73"/>
-      <c r="G34" s="74"/>
+      <c r="D34" s="68"/>
+      <c r="E34" s="68"/>
+      <c r="F34" s="68"/>
+      <c r="G34" s="69"/>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A35" s="82">
+      <c r="A35" s="84">
         <v>46210</v>
       </c>
-      <c r="B35" s="67" t="s">
+      <c r="B35" s="66" t="s">
         <v>5</v>
       </c>
-      <c r="C35" s="67" t="s">
+      <c r="C35" s="66" t="s">
         <v>46</v>
       </c>
-      <c r="D35" s="67"/>
-      <c r="E35" s="67"/>
-      <c r="F35" s="67"/>
-      <c r="G35" s="67"/>
+      <c r="D35" s="66"/>
+      <c r="E35" s="66"/>
+      <c r="F35" s="66"/>
+      <c r="G35" s="66"/>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A36" s="82"/>
-      <c r="B36" s="67"/>
-      <c r="C36" s="67" t="s">
+      <c r="A36" s="84"/>
+      <c r="B36" s="66"/>
+      <c r="C36" s="66" t="s">
         <v>27</v>
       </c>
-      <c r="D36" s="67"/>
-      <c r="E36" s="67"/>
-      <c r="F36" s="67"/>
-      <c r="G36" s="67"/>
+      <c r="D36" s="66"/>
+      <c r="E36" s="66"/>
+      <c r="F36" s="66"/>
+      <c r="G36" s="66"/>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A37" s="82"/>
-      <c r="B37" s="67"/>
-      <c r="C37" s="67" t="s">
+      <c r="A37" s="84"/>
+      <c r="B37" s="66"/>
+      <c r="C37" s="66" t="s">
         <v>47</v>
       </c>
-      <c r="D37" s="67"/>
-      <c r="E37" s="67"/>
-      <c r="F37" s="67"/>
-      <c r="G37" s="67"/>
+      <c r="D37" s="66"/>
+      <c r="E37" s="66"/>
+      <c r="F37" s="66"/>
+      <c r="G37" s="66"/>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A38" s="82"/>
-      <c r="B38" s="67" t="s">
-        <v>4</v>
-      </c>
-      <c r="C38" s="67" t="s">
+      <c r="A38" s="84"/>
+      <c r="B38" s="66" t="s">
+        <v>4</v>
+      </c>
+      <c r="C38" s="66" t="s">
         <v>52</v>
       </c>
-      <c r="D38" s="67"/>
-      <c r="E38" s="67"/>
-      <c r="F38" s="67"/>
-      <c r="G38" s="67"/>
+      <c r="D38" s="66"/>
+      <c r="E38" s="66"/>
+      <c r="F38" s="66"/>
+      <c r="G38" s="66"/>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A39" s="82"/>
-      <c r="B39" s="67"/>
-      <c r="C39" s="67" t="s">
+      <c r="A39" s="84"/>
+      <c r="B39" s="66"/>
+      <c r="C39" s="66" t="s">
         <v>53</v>
       </c>
-      <c r="D39" s="67"/>
-      <c r="E39" s="67"/>
-      <c r="F39" s="67"/>
-      <c r="G39" s="67"/>
+      <c r="D39" s="66"/>
+      <c r="E39" s="66"/>
+      <c r="F39" s="66"/>
+      <c r="G39" s="66"/>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A40" s="82"/>
-      <c r="B40" s="67"/>
-      <c r="C40" s="67" t="s">
+      <c r="A40" s="84"/>
+      <c r="B40" s="66"/>
+      <c r="C40" s="66" t="s">
         <v>48</v>
       </c>
-      <c r="D40" s="67"/>
-      <c r="E40" s="67"/>
-      <c r="F40" s="67"/>
-      <c r="G40" s="67"/>
+      <c r="D40" s="66"/>
+      <c r="E40" s="66"/>
+      <c r="F40" s="66"/>
+      <c r="G40" s="66"/>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A41" s="82"/>
-      <c r="B41" s="67"/>
-      <c r="C41" s="67" t="s">
+      <c r="A41" s="84"/>
+      <c r="B41" s="66"/>
+      <c r="C41" s="66" t="s">
         <v>49</v>
       </c>
-      <c r="D41" s="67"/>
-      <c r="E41" s="67"/>
-      <c r="F41" s="67"/>
-      <c r="G41" s="67"/>
+      <c r="D41" s="66"/>
+      <c r="E41" s="66"/>
+      <c r="F41" s="66"/>
+      <c r="G41" s="66"/>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A42" s="82"/>
-      <c r="B42" s="67"/>
-      <c r="C42" s="67" t="s">
+      <c r="A42" s="84"/>
+      <c r="B42" s="66"/>
+      <c r="C42" s="66" t="s">
         <v>50</v>
       </c>
-      <c r="D42" s="67"/>
-      <c r="E42" s="67"/>
-      <c r="F42" s="67"/>
-      <c r="G42" s="67"/>
+      <c r="D42" s="66"/>
+      <c r="E42" s="66"/>
+      <c r="F42" s="66"/>
+      <c r="G42" s="66"/>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A43" s="82"/>
-      <c r="B43" s="67"/>
-      <c r="C43" s="67" t="s">
+      <c r="A43" s="84"/>
+      <c r="B43" s="66"/>
+      <c r="C43" s="66" t="s">
         <v>51</v>
       </c>
-      <c r="D43" s="67"/>
-      <c r="E43" s="67"/>
-      <c r="F43" s="67"/>
-      <c r="G43" s="67"/>
+      <c r="D43" s="66"/>
+      <c r="E43" s="66"/>
+      <c r="F43" s="66"/>
+      <c r="G43" s="66"/>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A44" s="82"/>
-      <c r="B44" s="67"/>
-      <c r="C44" s="72" t="s">
+      <c r="A44" s="84"/>
+      <c r="B44" s="66"/>
+      <c r="C44" s="67" t="s">
         <v>54</v>
       </c>
-      <c r="D44" s="73"/>
-      <c r="E44" s="73"/>
-      <c r="F44" s="73"/>
-      <c r="G44" s="74"/>
+      <c r="D44" s="68"/>
+      <c r="E44" s="68"/>
+      <c r="F44" s="68"/>
+      <c r="G44" s="69"/>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A45" s="6">
@@ -2069,13 +2069,13 @@
       <c r="B45" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="C45" s="67" t="s">
+      <c r="C45" s="66" t="s">
         <v>55</v>
       </c>
-      <c r="D45" s="67"/>
-      <c r="E45" s="67"/>
-      <c r="F45" s="67"/>
-      <c r="G45" s="67"/>
+      <c r="D45" s="66"/>
+      <c r="E45" s="66"/>
+      <c r="F45" s="66"/>
+      <c r="G45" s="66"/>
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A46" s="6">
@@ -2084,255 +2084,255 @@
       <c r="B46" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="C46" s="67" t="s">
+      <c r="C46" s="66" t="s">
         <v>59</v>
       </c>
-      <c r="D46" s="67"/>
-      <c r="E46" s="67"/>
-      <c r="F46" s="67"/>
-      <c r="G46" s="67"/>
+      <c r="D46" s="66"/>
+      <c r="E46" s="66"/>
+      <c r="F46" s="66"/>
+      <c r="G46" s="66"/>
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A47" s="80">
+      <c r="A47" s="85">
         <v>46213</v>
       </c>
-      <c r="B47" s="78" t="s">
-        <v>4</v>
-      </c>
-      <c r="C47" s="72" t="s">
+      <c r="B47" s="75" t="s">
+        <v>4</v>
+      </c>
+      <c r="C47" s="67" t="s">
         <v>56</v>
       </c>
-      <c r="D47" s="73"/>
-      <c r="E47" s="73"/>
-      <c r="F47" s="73"/>
-      <c r="G47" s="74"/>
+      <c r="D47" s="68"/>
+      <c r="E47" s="68"/>
+      <c r="F47" s="68"/>
+      <c r="G47" s="69"/>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A48" s="83"/>
-      <c r="B48" s="86"/>
-      <c r="C48" s="72" t="s">
+      <c r="A48" s="86"/>
+      <c r="B48" s="77"/>
+      <c r="C48" s="67" t="s">
         <v>57</v>
       </c>
-      <c r="D48" s="73"/>
-      <c r="E48" s="73"/>
-      <c r="F48" s="73"/>
-      <c r="G48" s="74"/>
+      <c r="D48" s="68"/>
+      <c r="E48" s="68"/>
+      <c r="F48" s="68"/>
+      <c r="G48" s="69"/>
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A49" s="83"/>
-      <c r="B49" s="86"/>
-      <c r="C49" s="72" t="s">
+      <c r="A49" s="86"/>
+      <c r="B49" s="77"/>
+      <c r="C49" s="67" t="s">
         <v>58</v>
       </c>
-      <c r="D49" s="73"/>
-      <c r="E49" s="73"/>
-      <c r="F49" s="73"/>
-      <c r="G49" s="74"/>
+      <c r="D49" s="68"/>
+      <c r="E49" s="68"/>
+      <c r="F49" s="68"/>
+      <c r="G49" s="69"/>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A50" s="83"/>
-      <c r="B50" s="86"/>
-      <c r="C50" s="72" t="s">
+      <c r="A50" s="86"/>
+      <c r="B50" s="77"/>
+      <c r="C50" s="67" t="s">
         <v>60</v>
       </c>
-      <c r="D50" s="73"/>
-      <c r="E50" s="73"/>
-      <c r="F50" s="73"/>
-      <c r="G50" s="74"/>
+      <c r="D50" s="68"/>
+      <c r="E50" s="68"/>
+      <c r="F50" s="68"/>
+      <c r="G50" s="69"/>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A51" s="81"/>
-      <c r="B51" s="79"/>
-      <c r="C51" s="72" t="s">
+      <c r="A51" s="87"/>
+      <c r="B51" s="76"/>
+      <c r="C51" s="67" t="s">
         <v>61</v>
       </c>
-      <c r="D51" s="73"/>
-      <c r="E51" s="73"/>
-      <c r="F51" s="73"/>
-      <c r="G51" s="74"/>
+      <c r="D51" s="68"/>
+      <c r="E51" s="68"/>
+      <c r="F51" s="68"/>
+      <c r="G51" s="69"/>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A52" s="71">
+      <c r="A52" s="65">
         <v>46214</v>
       </c>
       <c r="B52" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="C52" s="67" t="s">
+      <c r="C52" s="66" t="s">
         <v>62</v>
       </c>
-      <c r="D52" s="67"/>
-      <c r="E52" s="67"/>
-      <c r="F52" s="67"/>
-      <c r="G52" s="67"/>
+      <c r="D52" s="66"/>
+      <c r="E52" s="66"/>
+      <c r="F52" s="66"/>
+      <c r="G52" s="66"/>
     </row>
     <row r="53" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A53" s="71"/>
+      <c r="A53" s="65"/>
       <c r="B53" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="C53" s="67" t="s">
+      <c r="C53" s="66" t="s">
         <v>63</v>
       </c>
-      <c r="D53" s="67"/>
-      <c r="E53" s="67"/>
-      <c r="F53" s="67"/>
-      <c r="G53" s="67"/>
+      <c r="D53" s="66"/>
+      <c r="E53" s="66"/>
+      <c r="F53" s="66"/>
+      <c r="G53" s="66"/>
     </row>
     <row r="54" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A54" s="71">
+      <c r="A54" s="65">
         <v>46216</v>
       </c>
       <c r="B54" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="C54" s="72" t="s">
+      <c r="C54" s="67" t="s">
         <v>70</v>
       </c>
-      <c r="D54" s="73"/>
-      <c r="E54" s="73"/>
-      <c r="F54" s="73"/>
-      <c r="G54" s="74"/>
+      <c r="D54" s="68"/>
+      <c r="E54" s="68"/>
+      <c r="F54" s="68"/>
+      <c r="G54" s="69"/>
     </row>
     <row r="55" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A55" s="71"/>
-      <c r="B55" s="67" t="s">
-        <v>4</v>
-      </c>
-      <c r="C55" s="85" t="s">
+      <c r="A55" s="65"/>
+      <c r="B55" s="66" t="s">
+        <v>4</v>
+      </c>
+      <c r="C55" s="89" t="s">
         <v>65</v>
       </c>
-      <c r="D55" s="85"/>
-      <c r="E55" s="85"/>
-      <c r="F55" s="85"/>
-      <c r="G55" s="85"/>
+      <c r="D55" s="89"/>
+      <c r="E55" s="89"/>
+      <c r="F55" s="89"/>
+      <c r="G55" s="89"/>
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A56" s="71"/>
-      <c r="B56" s="67"/>
-      <c r="C56" s="85" t="s">
+      <c r="A56" s="65"/>
+      <c r="B56" s="66"/>
+      <c r="C56" s="89" t="s">
         <v>66</v>
       </c>
-      <c r="D56" s="85"/>
-      <c r="E56" s="85"/>
-      <c r="F56" s="85"/>
-      <c r="G56" s="85"/>
+      <c r="D56" s="89"/>
+      <c r="E56" s="89"/>
+      <c r="F56" s="89"/>
+      <c r="G56" s="89"/>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A57" s="71"/>
-      <c r="B57" s="67"/>
-      <c r="C57" s="85" t="s">
+      <c r="A57" s="65"/>
+      <c r="B57" s="66"/>
+      <c r="C57" s="89" t="s">
         <v>67</v>
       </c>
-      <c r="D57" s="85"/>
-      <c r="E57" s="85"/>
-      <c r="F57" s="85"/>
-      <c r="G57" s="85"/>
+      <c r="D57" s="89"/>
+      <c r="E57" s="89"/>
+      <c r="F57" s="89"/>
+      <c r="G57" s="89"/>
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A58" s="71"/>
-      <c r="B58" s="67"/>
-      <c r="C58" s="85" t="s">
+      <c r="A58" s="65"/>
+      <c r="B58" s="66"/>
+      <c r="C58" s="89" t="s">
         <v>68</v>
       </c>
-      <c r="D58" s="85"/>
-      <c r="E58" s="85"/>
-      <c r="F58" s="85"/>
-      <c r="G58" s="85"/>
+      <c r="D58" s="89"/>
+      <c r="E58" s="89"/>
+      <c r="F58" s="89"/>
+      <c r="G58" s="89"/>
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A59" s="71"/>
-      <c r="B59" s="67"/>
-      <c r="C59" s="85" t="s">
+      <c r="A59" s="65"/>
+      <c r="B59" s="66"/>
+      <c r="C59" s="89" t="s">
         <v>69</v>
       </c>
-      <c r="D59" s="85"/>
-      <c r="E59" s="85"/>
-      <c r="F59" s="85"/>
-      <c r="G59" s="85"/>
+      <c r="D59" s="89"/>
+      <c r="E59" s="89"/>
+      <c r="F59" s="89"/>
+      <c r="G59" s="89"/>
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A60" s="71"/>
-      <c r="B60" s="67"/>
-      <c r="C60" s="85" t="s">
+      <c r="A60" s="65"/>
+      <c r="B60" s="66"/>
+      <c r="C60" s="89" t="s">
         <v>64</v>
       </c>
-      <c r="D60" s="85"/>
-      <c r="E60" s="85"/>
-      <c r="F60" s="85"/>
-      <c r="G60" s="85"/>
+      <c r="D60" s="89"/>
+      <c r="E60" s="89"/>
+      <c r="F60" s="89"/>
+      <c r="G60" s="89"/>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A61" s="71"/>
-      <c r="B61" s="67"/>
-      <c r="C61" s="85" t="s">
+      <c r="A61" s="65"/>
+      <c r="B61" s="66"/>
+      <c r="C61" s="89" t="s">
         <v>71</v>
       </c>
-      <c r="D61" s="85"/>
-      <c r="E61" s="85"/>
-      <c r="F61" s="85"/>
-      <c r="G61" s="85"/>
+      <c r="D61" s="89"/>
+      <c r="E61" s="89"/>
+      <c r="F61" s="89"/>
+      <c r="G61" s="89"/>
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A62" s="71"/>
-      <c r="B62" s="67"/>
-      <c r="C62" s="85" t="s">
+      <c r="A62" s="65"/>
+      <c r="B62" s="66"/>
+      <c r="C62" s="89" t="s">
         <v>72</v>
       </c>
-      <c r="D62" s="85"/>
-      <c r="E62" s="85"/>
-      <c r="F62" s="85"/>
-      <c r="G62" s="85"/>
+      <c r="D62" s="89"/>
+      <c r="E62" s="89"/>
+      <c r="F62" s="89"/>
+      <c r="G62" s="89"/>
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A63" s="71"/>
-      <c r="B63" s="67"/>
-      <c r="C63" s="85" t="s">
+      <c r="A63" s="65"/>
+      <c r="B63" s="66"/>
+      <c r="C63" s="89" t="s">
         <v>73</v>
       </c>
-      <c r="D63" s="85"/>
-      <c r="E63" s="85"/>
-      <c r="F63" s="85"/>
-      <c r="G63" s="85"/>
+      <c r="D63" s="89"/>
+      <c r="E63" s="89"/>
+      <c r="F63" s="89"/>
+      <c r="G63" s="89"/>
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A64" s="71">
+      <c r="A64" s="65">
         <v>46217</v>
       </c>
       <c r="B64" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="C64" s="67" t="s">
+      <c r="C64" s="66" t="s">
         <v>15</v>
       </c>
-      <c r="D64" s="67"/>
-      <c r="E64" s="67"/>
-      <c r="F64" s="67"/>
-      <c r="G64" s="67"/>
+      <c r="D64" s="66"/>
+      <c r="E64" s="66"/>
+      <c r="F64" s="66"/>
+      <c r="G64" s="66"/>
     </row>
     <row r="65" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A65" s="71"/>
-      <c r="B65" s="67" t="s">
-        <v>4</v>
-      </c>
-      <c r="C65" s="67" t="s">
+      <c r="A65" s="65"/>
+      <c r="B65" s="66" t="s">
+        <v>4</v>
+      </c>
+      <c r="C65" s="66" t="s">
         <v>39</v>
       </c>
-      <c r="D65" s="67"/>
-      <c r="E65" s="67"/>
-      <c r="F65" s="67"/>
-      <c r="G65" s="67"/>
+      <c r="D65" s="66"/>
+      <c r="E65" s="66"/>
+      <c r="F65" s="66"/>
+      <c r="G65" s="66"/>
     </row>
     <row r="66" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A66" s="71"/>
-      <c r="B66" s="67"/>
-      <c r="C66" s="67" t="s">
+      <c r="A66" s="65"/>
+      <c r="B66" s="66"/>
+      <c r="C66" s="66" t="s">
         <v>74</v>
       </c>
-      <c r="D66" s="67"/>
-      <c r="E66" s="67"/>
-      <c r="F66" s="67"/>
-      <c r="G66" s="67"/>
+      <c r="D66" s="66"/>
+      <c r="E66" s="66"/>
+      <c r="F66" s="66"/>
+      <c r="G66" s="66"/>
     </row>
     <row r="67" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A67" s="6">
@@ -2341,164 +2341,164 @@
       <c r="B67" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="C67" s="67" t="s">
+      <c r="C67" s="66" t="s">
         <v>75</v>
       </c>
-      <c r="D67" s="67"/>
-      <c r="E67" s="67"/>
-      <c r="F67" s="67"/>
-      <c r="G67" s="67"/>
+      <c r="D67" s="66"/>
+      <c r="E67" s="66"/>
+      <c r="F67" s="66"/>
+      <c r="G67" s="66"/>
     </row>
     <row r="68" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A68" s="71">
+      <c r="A68" s="65">
         <v>46220</v>
       </c>
-      <c r="B68" s="67" t="s">
-        <v>4</v>
-      </c>
-      <c r="C68" s="67" t="s">
+      <c r="B68" s="66" t="s">
+        <v>4</v>
+      </c>
+      <c r="C68" s="66" t="s">
         <v>76</v>
       </c>
-      <c r="D68" s="67"/>
-      <c r="E68" s="67"/>
-      <c r="F68" s="67"/>
-      <c r="G68" s="67"/>
+      <c r="D68" s="66"/>
+      <c r="E68" s="66"/>
+      <c r="F68" s="66"/>
+      <c r="G68" s="66"/>
     </row>
     <row r="69" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A69" s="71"/>
-      <c r="B69" s="67"/>
-      <c r="C69" s="67" t="s">
+      <c r="A69" s="65"/>
+      <c r="B69" s="66"/>
+      <c r="C69" s="66" t="s">
         <v>77</v>
       </c>
-      <c r="D69" s="67"/>
-      <c r="E69" s="67"/>
-      <c r="F69" s="67"/>
-      <c r="G69" s="67"/>
+      <c r="D69" s="66"/>
+      <c r="E69" s="66"/>
+      <c r="F69" s="66"/>
+      <c r="G69" s="66"/>
     </row>
     <row r="70" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A70" s="71">
+      <c r="A70" s="65">
         <v>46223</v>
       </c>
-      <c r="B70" s="67" t="s">
-        <v>4</v>
-      </c>
-      <c r="C70" s="72" t="s">
+      <c r="B70" s="66" t="s">
+        <v>4</v>
+      </c>
+      <c r="C70" s="67" t="s">
         <v>78</v>
       </c>
-      <c r="D70" s="73"/>
-      <c r="E70" s="73"/>
-      <c r="F70" s="73"/>
-      <c r="G70" s="74"/>
+      <c r="D70" s="68"/>
+      <c r="E70" s="68"/>
+      <c r="F70" s="68"/>
+      <c r="G70" s="69"/>
     </row>
     <row r="71" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A71" s="71"/>
-      <c r="B71" s="67"/>
-      <c r="C71" s="72" t="s">
+      <c r="A71" s="65"/>
+      <c r="B71" s="66"/>
+      <c r="C71" s="67" t="s">
         <v>79</v>
       </c>
-      <c r="D71" s="73"/>
-      <c r="E71" s="73"/>
-      <c r="F71" s="73"/>
-      <c r="G71" s="74"/>
+      <c r="D71" s="68"/>
+      <c r="E71" s="68"/>
+      <c r="F71" s="68"/>
+      <c r="G71" s="69"/>
     </row>
     <row r="72" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A72" s="71"/>
-      <c r="B72" s="67"/>
-      <c r="C72" s="72" t="s">
+      <c r="A72" s="65"/>
+      <c r="B72" s="66"/>
+      <c r="C72" s="67" t="s">
         <v>80</v>
       </c>
-      <c r="D72" s="73"/>
-      <c r="E72" s="73"/>
-      <c r="F72" s="73"/>
-      <c r="G72" s="74"/>
+      <c r="D72" s="68"/>
+      <c r="E72" s="68"/>
+      <c r="F72" s="68"/>
+      <c r="G72" s="69"/>
     </row>
     <row r="73" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A73" s="71"/>
-      <c r="B73" s="67"/>
-      <c r="C73" s="72" t="s">
+      <c r="A73" s="65"/>
+      <c r="B73" s="66"/>
+      <c r="C73" s="67" t="s">
         <v>81</v>
       </c>
-      <c r="D73" s="73"/>
-      <c r="E73" s="73"/>
-      <c r="F73" s="73"/>
-      <c r="G73" s="74"/>
+      <c r="D73" s="68"/>
+      <c r="E73" s="68"/>
+      <c r="F73" s="68"/>
+      <c r="G73" s="69"/>
     </row>
     <row r="74" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A74" s="71"/>
-      <c r="B74" s="67"/>
-      <c r="C74" s="72" t="s">
+      <c r="A74" s="65"/>
+      <c r="B74" s="66"/>
+      <c r="C74" s="67" t="s">
         <v>39</v>
       </c>
-      <c r="D74" s="73"/>
-      <c r="E74" s="73"/>
-      <c r="F74" s="73"/>
-      <c r="G74" s="74"/>
+      <c r="D74" s="68"/>
+      <c r="E74" s="68"/>
+      <c r="F74" s="68"/>
+      <c r="G74" s="69"/>
     </row>
     <row r="75" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A75" s="71"/>
-      <c r="B75" s="67"/>
-      <c r="C75" s="72" t="s">
+      <c r="A75" s="65"/>
+      <c r="B75" s="66"/>
+      <c r="C75" s="67" t="s">
         <v>82</v>
       </c>
-      <c r="D75" s="73"/>
-      <c r="E75" s="73"/>
-      <c r="F75" s="73"/>
-      <c r="G75" s="74"/>
+      <c r="D75" s="68"/>
+      <c r="E75" s="68"/>
+      <c r="F75" s="68"/>
+      <c r="G75" s="69"/>
     </row>
     <row r="76" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A76" s="71"/>
-      <c r="B76" s="67"/>
-      <c r="C76" s="72" t="s">
+      <c r="A76" s="65"/>
+      <c r="B76" s="66"/>
+      <c r="C76" s="67" t="s">
         <v>72</v>
       </c>
-      <c r="D76" s="73"/>
-      <c r="E76" s="73"/>
-      <c r="F76" s="73"/>
-      <c r="G76" s="74"/>
+      <c r="D76" s="68"/>
+      <c r="E76" s="68"/>
+      <c r="F76" s="68"/>
+      <c r="G76" s="69"/>
     </row>
     <row r="77" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A77" s="71"/>
-      <c r="B77" s="67"/>
-      <c r="C77" s="68" t="s">
+      <c r="A77" s="65"/>
+      <c r="B77" s="66"/>
+      <c r="C77" s="62" t="s">
         <v>83</v>
       </c>
-      <c r="D77" s="69"/>
-      <c r="E77" s="69"/>
-      <c r="F77" s="69"/>
-      <c r="G77" s="70"/>
+      <c r="D77" s="63"/>
+      <c r="E77" s="63"/>
+      <c r="F77" s="63"/>
+      <c r="G77" s="64"/>
     </row>
     <row r="78" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A78" s="71"/>
-      <c r="B78" s="67"/>
-      <c r="C78" s="68" t="s">
+      <c r="A78" s="65"/>
+      <c r="B78" s="66"/>
+      <c r="C78" s="62" t="s">
         <v>84</v>
       </c>
-      <c r="D78" s="69"/>
-      <c r="E78" s="69"/>
-      <c r="F78" s="69"/>
-      <c r="G78" s="70"/>
+      <c r="D78" s="63"/>
+      <c r="E78" s="63"/>
+      <c r="F78" s="63"/>
+      <c r="G78" s="64"/>
     </row>
     <row r="79" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A79" s="71"/>
-      <c r="B79" s="67"/>
-      <c r="C79" s="68" t="s">
+      <c r="A79" s="65"/>
+      <c r="B79" s="66"/>
+      <c r="C79" s="62" t="s">
         <v>85</v>
       </c>
-      <c r="D79" s="69"/>
-      <c r="E79" s="69"/>
-      <c r="F79" s="69"/>
-      <c r="G79" s="70"/>
+      <c r="D79" s="63"/>
+      <c r="E79" s="63"/>
+      <c r="F79" s="63"/>
+      <c r="G79" s="64"/>
     </row>
     <row r="80" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A80" s="71"/>
-      <c r="B80" s="67"/>
-      <c r="C80" s="68" t="s">
+      <c r="A80" s="65"/>
+      <c r="B80" s="66"/>
+      <c r="C80" s="62" t="s">
         <v>86</v>
       </c>
-      <c r="D80" s="69"/>
-      <c r="E80" s="69"/>
-      <c r="F80" s="69"/>
-      <c r="G80" s="70"/>
+      <c r="D80" s="63"/>
+      <c r="E80" s="63"/>
+      <c r="F80" s="63"/>
+      <c r="G80" s="64"/>
     </row>
     <row r="81" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A81" s="6">
@@ -2507,353 +2507,353 @@
       <c r="B81" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="C81" s="67" t="s">
+      <c r="C81" s="66" t="s">
         <v>87</v>
       </c>
-      <c r="D81" s="67"/>
-      <c r="E81" s="67"/>
-      <c r="F81" s="67"/>
-      <c r="G81" s="67"/>
+      <c r="D81" s="66"/>
+      <c r="E81" s="66"/>
+      <c r="F81" s="66"/>
+      <c r="G81" s="66"/>
     </row>
     <row r="82" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A82" s="71">
+      <c r="A82" s="65">
         <v>46225</v>
       </c>
-      <c r="B82" s="67" t="s">
+      <c r="B82" s="66" t="s">
         <v>5</v>
       </c>
-      <c r="C82" s="67" t="s">
+      <c r="C82" s="66" t="s">
         <v>91</v>
       </c>
-      <c r="D82" s="67"/>
-      <c r="E82" s="67"/>
-      <c r="F82" s="67"/>
-      <c r="G82" s="67"/>
+      <c r="D82" s="66"/>
+      <c r="E82" s="66"/>
+      <c r="F82" s="66"/>
+      <c r="G82" s="66"/>
     </row>
     <row r="83" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A83" s="71"/>
-      <c r="B83" s="67"/>
-      <c r="C83" s="67" t="s">
+      <c r="A83" s="65"/>
+      <c r="B83" s="66"/>
+      <c r="C83" s="66" t="s">
         <v>90</v>
       </c>
-      <c r="D83" s="67"/>
-      <c r="E83" s="67"/>
-      <c r="F83" s="67"/>
-      <c r="G83" s="67"/>
+      <c r="D83" s="66"/>
+      <c r="E83" s="66"/>
+      <c r="F83" s="66"/>
+      <c r="G83" s="66"/>
     </row>
     <row r="84" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A84" s="71"/>
-      <c r="B84" s="67"/>
-      <c r="C84" s="67" t="s">
+      <c r="A84" s="65"/>
+      <c r="B84" s="66"/>
+      <c r="C84" s="66" t="s">
         <v>93</v>
       </c>
-      <c r="D84" s="67"/>
-      <c r="E84" s="67"/>
-      <c r="F84" s="67"/>
-      <c r="G84" s="67"/>
+      <c r="D84" s="66"/>
+      <c r="E84" s="66"/>
+      <c r="F84" s="66"/>
+      <c r="G84" s="66"/>
     </row>
     <row r="85" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A85" s="71"/>
-      <c r="B85" s="67" t="s">
-        <v>4</v>
-      </c>
-      <c r="C85" s="67" t="s">
+      <c r="A85" s="65"/>
+      <c r="B85" s="66" t="s">
+        <v>4</v>
+      </c>
+      <c r="C85" s="66" t="s">
         <v>88</v>
       </c>
-      <c r="D85" s="67"/>
-      <c r="E85" s="67"/>
-      <c r="F85" s="67"/>
-      <c r="G85" s="67"/>
+      <c r="D85" s="66"/>
+      <c r="E85" s="66"/>
+      <c r="F85" s="66"/>
+      <c r="G85" s="66"/>
     </row>
     <row r="86" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A86" s="71"/>
-      <c r="B86" s="67"/>
-      <c r="C86" s="67" t="s">
+      <c r="A86" s="65"/>
+      <c r="B86" s="66"/>
+      <c r="C86" s="66" t="s">
         <v>72</v>
       </c>
-      <c r="D86" s="67"/>
-      <c r="E86" s="67"/>
-      <c r="F86" s="67"/>
-      <c r="G86" s="67"/>
+      <c r="D86" s="66"/>
+      <c r="E86" s="66"/>
+      <c r="F86" s="66"/>
+      <c r="G86" s="66"/>
     </row>
     <row r="87" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A87" s="71"/>
-      <c r="B87" s="67"/>
-      <c r="C87" s="67" t="s">
+      <c r="A87" s="65"/>
+      <c r="B87" s="66"/>
+      <c r="C87" s="66" t="s">
         <v>89</v>
       </c>
-      <c r="D87" s="67"/>
-      <c r="E87" s="67"/>
-      <c r="F87" s="67"/>
-      <c r="G87" s="67"/>
+      <c r="D87" s="66"/>
+      <c r="E87" s="66"/>
+      <c r="F87" s="66"/>
+      <c r="G87" s="66"/>
     </row>
     <row r="88" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A88" s="71"/>
-      <c r="B88" s="67"/>
-      <c r="C88" s="67" t="s">
+      <c r="A88" s="65"/>
+      <c r="B88" s="66"/>
+      <c r="C88" s="66" t="s">
         <v>35</v>
       </c>
-      <c r="D88" s="67"/>
-      <c r="E88" s="67"/>
-      <c r="F88" s="67"/>
-      <c r="G88" s="67"/>
+      <c r="D88" s="66"/>
+      <c r="E88" s="66"/>
+      <c r="F88" s="66"/>
+      <c r="G88" s="66"/>
     </row>
     <row r="89" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A89" s="71"/>
-      <c r="B89" s="67"/>
-      <c r="C89" s="72" t="s">
+      <c r="A89" s="65"/>
+      <c r="B89" s="66"/>
+      <c r="C89" s="67" t="s">
         <v>39</v>
       </c>
-      <c r="D89" s="73"/>
-      <c r="E89" s="73"/>
-      <c r="F89" s="73"/>
-      <c r="G89" s="74"/>
+      <c r="D89" s="68"/>
+      <c r="E89" s="68"/>
+      <c r="F89" s="68"/>
+      <c r="G89" s="69"/>
     </row>
     <row r="90" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A90" s="71"/>
-      <c r="B90" s="67"/>
-      <c r="C90" s="67" t="s">
+      <c r="A90" s="65"/>
+      <c r="B90" s="66"/>
+      <c r="C90" s="66" t="s">
         <v>92</v>
       </c>
-      <c r="D90" s="67"/>
-      <c r="E90" s="67"/>
-      <c r="F90" s="67"/>
-      <c r="G90" s="67"/>
+      <c r="D90" s="66"/>
+      <c r="E90" s="66"/>
+      <c r="F90" s="66"/>
+      <c r="G90" s="66"/>
     </row>
     <row r="91" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A91" s="80">
+      <c r="A91" s="85">
         <v>46227</v>
       </c>
-      <c r="B91" s="78" t="s">
+      <c r="B91" s="75" t="s">
         <v>5</v>
       </c>
-      <c r="C91" s="67" t="s">
+      <c r="C91" s="66" t="s">
         <v>94</v>
       </c>
-      <c r="D91" s="67"/>
-      <c r="E91" s="67"/>
-      <c r="F91" s="67"/>
-      <c r="G91" s="67"/>
+      <c r="D91" s="66"/>
+      <c r="E91" s="66"/>
+      <c r="F91" s="66"/>
+      <c r="G91" s="66"/>
     </row>
     <row r="92" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A92" s="81"/>
-      <c r="B92" s="79"/>
-      <c r="C92" s="72" t="s">
+      <c r="A92" s="87"/>
+      <c r="B92" s="76"/>
+      <c r="C92" s="67" t="s">
         <v>95</v>
       </c>
-      <c r="D92" s="73"/>
-      <c r="E92" s="73"/>
-      <c r="F92" s="73"/>
-      <c r="G92" s="74"/>
+      <c r="D92" s="68"/>
+      <c r="E92" s="68"/>
+      <c r="F92" s="68"/>
+      <c r="G92" s="69"/>
     </row>
     <row r="93" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A93" s="71">
+      <c r="A93" s="65">
         <v>46228</v>
       </c>
-      <c r="B93" s="67" t="s">
-        <v>4</v>
-      </c>
-      <c r="C93" s="67" t="s">
+      <c r="B93" s="66" t="s">
+        <v>4</v>
+      </c>
+      <c r="C93" s="66" t="s">
         <v>96</v>
       </c>
-      <c r="D93" s="67"/>
-      <c r="E93" s="67"/>
-      <c r="F93" s="67"/>
-      <c r="G93" s="67"/>
+      <c r="D93" s="66"/>
+      <c r="E93" s="66"/>
+      <c r="F93" s="66"/>
+      <c r="G93" s="66"/>
     </row>
     <row r="94" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A94" s="71"/>
-      <c r="B94" s="67"/>
-      <c r="C94" s="67" t="s">
+      <c r="A94" s="65"/>
+      <c r="B94" s="66"/>
+      <c r="C94" s="66" t="s">
         <v>97</v>
       </c>
-      <c r="D94" s="67"/>
-      <c r="E94" s="67"/>
-      <c r="F94" s="67"/>
-      <c r="G94" s="67"/>
+      <c r="D94" s="66"/>
+      <c r="E94" s="66"/>
+      <c r="F94" s="66"/>
+      <c r="G94" s="66"/>
     </row>
     <row r="95" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A95" s="71"/>
-      <c r="B95" s="67"/>
-      <c r="C95" s="67" t="s">
+      <c r="A95" s="65"/>
+      <c r="B95" s="66"/>
+      <c r="C95" s="66" t="s">
         <v>98</v>
       </c>
-      <c r="D95" s="67"/>
-      <c r="E95" s="67"/>
-      <c r="F95" s="67"/>
-      <c r="G95" s="67"/>
+      <c r="D95" s="66"/>
+      <c r="E95" s="66"/>
+      <c r="F95" s="66"/>
+      <c r="G95" s="66"/>
     </row>
     <row r="96" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A96" s="71"/>
-      <c r="B96" s="67"/>
-      <c r="C96" s="67" t="s">
+      <c r="A96" s="65"/>
+      <c r="B96" s="66"/>
+      <c r="C96" s="66" t="s">
         <v>99</v>
       </c>
-      <c r="D96" s="67"/>
-      <c r="E96" s="67"/>
-      <c r="F96" s="67"/>
-      <c r="G96" s="67"/>
+      <c r="D96" s="66"/>
+      <c r="E96" s="66"/>
+      <c r="F96" s="66"/>
+      <c r="G96" s="66"/>
     </row>
     <row r="97" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A97" s="71"/>
-      <c r="B97" s="67"/>
-      <c r="C97" s="67" t="s">
+      <c r="A97" s="65"/>
+      <c r="B97" s="66"/>
+      <c r="C97" s="66" t="s">
         <v>100</v>
       </c>
-      <c r="D97" s="67"/>
-      <c r="E97" s="67"/>
-      <c r="F97" s="67"/>
-      <c r="G97" s="67"/>
+      <c r="D97" s="66"/>
+      <c r="E97" s="66"/>
+      <c r="F97" s="66"/>
+      <c r="G97" s="66"/>
     </row>
     <row r="98" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A98" s="71"/>
-      <c r="B98" s="67"/>
-      <c r="C98" s="67" t="s">
+      <c r="A98" s="65"/>
+      <c r="B98" s="66"/>
+      <c r="C98" s="66" t="s">
         <v>101</v>
       </c>
-      <c r="D98" s="67"/>
-      <c r="E98" s="67"/>
-      <c r="F98" s="67"/>
-      <c r="G98" s="67"/>
+      <c r="D98" s="66"/>
+      <c r="E98" s="66"/>
+      <c r="F98" s="66"/>
+      <c r="G98" s="66"/>
     </row>
     <row r="99" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A99" s="71">
+      <c r="A99" s="65">
         <v>46230</v>
       </c>
-      <c r="B99" s="67" t="s">
-        <v>4</v>
-      </c>
-      <c r="C99" s="67" t="s">
+      <c r="B99" s="66" t="s">
+        <v>4</v>
+      </c>
+      <c r="C99" s="66" t="s">
         <v>102</v>
       </c>
-      <c r="D99" s="67"/>
-      <c r="E99" s="67"/>
-      <c r="F99" s="67"/>
-      <c r="G99" s="67"/>
+      <c r="D99" s="66"/>
+      <c r="E99" s="66"/>
+      <c r="F99" s="66"/>
+      <c r="G99" s="66"/>
     </row>
     <row r="100" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A100" s="71"/>
-      <c r="B100" s="67"/>
-      <c r="C100" s="67" t="s">
+      <c r="A100" s="65"/>
+      <c r="B100" s="66"/>
+      <c r="C100" s="66" t="s">
         <v>39</v>
       </c>
-      <c r="D100" s="67"/>
-      <c r="E100" s="67"/>
-      <c r="F100" s="67"/>
-      <c r="G100" s="67"/>
+      <c r="D100" s="66"/>
+      <c r="E100" s="66"/>
+      <c r="F100" s="66"/>
+      <c r="G100" s="66"/>
     </row>
     <row r="101" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A101" s="71">
+      <c r="A101" s="65">
         <v>46231</v>
       </c>
       <c r="B101" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="C101" s="77" t="s">
+      <c r="C101" s="91" t="s">
         <v>104</v>
       </c>
-      <c r="D101" s="77"/>
-      <c r="E101" s="77"/>
-      <c r="F101" s="77"/>
-      <c r="G101" s="77"/>
+      <c r="D101" s="91"/>
+      <c r="E101" s="91"/>
+      <c r="F101" s="91"/>
+      <c r="G101" s="91"/>
     </row>
     <row r="102" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A102" s="71"/>
+      <c r="A102" s="65"/>
       <c r="B102" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="C102" s="77" t="s">
+      <c r="C102" s="91" t="s">
         <v>103</v>
       </c>
-      <c r="D102" s="77"/>
-      <c r="E102" s="77"/>
-      <c r="F102" s="77"/>
-      <c r="G102" s="77"/>
+      <c r="D102" s="91"/>
+      <c r="E102" s="91"/>
+      <c r="F102" s="91"/>
+      <c r="G102" s="91"/>
     </row>
     <row r="103" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A103" s="75" t="s">
+      <c r="A103" s="90" t="s">
         <v>105</v>
       </c>
-      <c r="B103" s="67" t="s">
-        <v>4</v>
-      </c>
-      <c r="C103" s="76" t="s">
+      <c r="B103" s="66" t="s">
+        <v>4</v>
+      </c>
+      <c r="C103" s="80" t="s">
         <v>106</v>
       </c>
-      <c r="D103" s="76"/>
-      <c r="E103" s="76"/>
-      <c r="F103" s="76"/>
-      <c r="G103" s="76"/>
+      <c r="D103" s="80"/>
+      <c r="E103" s="80"/>
+      <c r="F103" s="80"/>
+      <c r="G103" s="80"/>
     </row>
     <row r="104" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A104" s="75"/>
-      <c r="B104" s="67"/>
-      <c r="C104" s="67" t="s">
+      <c r="A104" s="90"/>
+      <c r="B104" s="66"/>
+      <c r="C104" s="66" t="s">
         <v>86</v>
       </c>
-      <c r="D104" s="67"/>
-      <c r="E104" s="67"/>
-      <c r="F104" s="67"/>
-      <c r="G104" s="67"/>
+      <c r="D104" s="66"/>
+      <c r="E104" s="66"/>
+      <c r="F104" s="66"/>
+      <c r="G104" s="66"/>
     </row>
     <row r="105" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A105" s="75"/>
-      <c r="B105" s="67"/>
-      <c r="C105" s="67" t="s">
+      <c r="A105" s="90"/>
+      <c r="B105" s="66"/>
+      <c r="C105" s="66" t="s">
         <v>60</v>
       </c>
-      <c r="D105" s="67"/>
-      <c r="E105" s="67"/>
-      <c r="F105" s="67"/>
-      <c r="G105" s="67"/>
+      <c r="D105" s="66"/>
+      <c r="E105" s="66"/>
+      <c r="F105" s="66"/>
+      <c r="G105" s="66"/>
     </row>
     <row r="106" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A106" s="75"/>
-      <c r="B106" s="67"/>
-      <c r="C106" s="67" t="s">
+      <c r="A106" s="90"/>
+      <c r="B106" s="66"/>
+      <c r="C106" s="66" t="s">
         <v>50</v>
       </c>
-      <c r="D106" s="67"/>
-      <c r="E106" s="67"/>
-      <c r="F106" s="67"/>
-      <c r="G106" s="67"/>
+      <c r="D106" s="66"/>
+      <c r="E106" s="66"/>
+      <c r="F106" s="66"/>
+      <c r="G106" s="66"/>
     </row>
     <row r="107" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A107" s="75"/>
-      <c r="B107" s="67"/>
-      <c r="C107" s="67" t="s">
+      <c r="A107" s="90"/>
+      <c r="B107" s="66"/>
+      <c r="C107" s="66" t="s">
         <v>107</v>
       </c>
-      <c r="D107" s="67"/>
-      <c r="E107" s="67"/>
-      <c r="F107" s="67"/>
-      <c r="G107" s="67"/>
+      <c r="D107" s="66"/>
+      <c r="E107" s="66"/>
+      <c r="F107" s="66"/>
+      <c r="G107" s="66"/>
     </row>
     <row r="108" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A108" s="71">
+      <c r="A108" s="65">
         <v>46234</v>
       </c>
-      <c r="B108" s="67" t="s">
-        <v>4</v>
-      </c>
-      <c r="C108" s="67" t="s">
+      <c r="B108" s="66" t="s">
+        <v>4</v>
+      </c>
+      <c r="C108" s="66" t="s">
         <v>108</v>
       </c>
-      <c r="D108" s="67"/>
-      <c r="E108" s="67"/>
-      <c r="F108" s="67"/>
-      <c r="G108" s="67"/>
+      <c r="D108" s="66"/>
+      <c r="E108" s="66"/>
+      <c r="F108" s="66"/>
+      <c r="G108" s="66"/>
     </row>
     <row r="109" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A109" s="71"/>
-      <c r="B109" s="67"/>
-      <c r="C109" s="67" t="s">
+      <c r="A109" s="65"/>
+      <c r="B109" s="66"/>
+      <c r="C109" s="66" t="s">
         <v>39</v>
       </c>
-      <c r="D109" s="67"/>
-      <c r="E109" s="67"/>
-      <c r="F109" s="67"/>
-      <c r="G109" s="67"/>
+      <c r="D109" s="66"/>
+      <c r="E109" s="66"/>
+      <c r="F109" s="66"/>
+      <c r="G109" s="66"/>
     </row>
     <row r="110" spans="1:7" x14ac:dyDescent="0.25">
       <c r="D110" s="10"/>
@@ -2863,6 +2863,129 @@
     </row>
   </sheetData>
   <mergeCells count="147">
+    <mergeCell ref="A103:A107"/>
+    <mergeCell ref="B103:B107"/>
+    <mergeCell ref="C103:G103"/>
+    <mergeCell ref="C104:G104"/>
+    <mergeCell ref="C105:G105"/>
+    <mergeCell ref="C106:G106"/>
+    <mergeCell ref="C107:G107"/>
+    <mergeCell ref="A99:A100"/>
+    <mergeCell ref="B99:B100"/>
+    <mergeCell ref="C99:G99"/>
+    <mergeCell ref="C100:G100"/>
+    <mergeCell ref="C101:G101"/>
+    <mergeCell ref="C102:G102"/>
+    <mergeCell ref="A101:A102"/>
+    <mergeCell ref="B93:B98"/>
+    <mergeCell ref="A93:A98"/>
+    <mergeCell ref="C93:G93"/>
+    <mergeCell ref="C94:G94"/>
+    <mergeCell ref="C95:G95"/>
+    <mergeCell ref="C96:G96"/>
+    <mergeCell ref="C97:G97"/>
+    <mergeCell ref="C98:G98"/>
+    <mergeCell ref="C91:G91"/>
+    <mergeCell ref="C92:G92"/>
+    <mergeCell ref="B91:B92"/>
+    <mergeCell ref="A91:A92"/>
+    <mergeCell ref="A82:A90"/>
+    <mergeCell ref="B82:B84"/>
+    <mergeCell ref="C89:G89"/>
+    <mergeCell ref="C82:G82"/>
+    <mergeCell ref="C83:G83"/>
+    <mergeCell ref="C84:G84"/>
+    <mergeCell ref="C85:G85"/>
+    <mergeCell ref="C86:G86"/>
+    <mergeCell ref="C87:G87"/>
+    <mergeCell ref="C88:G88"/>
+    <mergeCell ref="C90:G90"/>
+    <mergeCell ref="B85:B90"/>
+    <mergeCell ref="C68:G68"/>
+    <mergeCell ref="C69:G69"/>
+    <mergeCell ref="A68:A69"/>
+    <mergeCell ref="B68:B69"/>
+    <mergeCell ref="A64:A66"/>
+    <mergeCell ref="C65:G65"/>
+    <mergeCell ref="C66:G66"/>
+    <mergeCell ref="B65:B66"/>
+    <mergeCell ref="C67:G67"/>
+    <mergeCell ref="C64:G64"/>
+    <mergeCell ref="C81:G81"/>
+    <mergeCell ref="B70:B80"/>
+    <mergeCell ref="A70:A80"/>
+    <mergeCell ref="C70:G70"/>
+    <mergeCell ref="C71:G71"/>
+    <mergeCell ref="C72:G72"/>
+    <mergeCell ref="C73:G73"/>
+    <mergeCell ref="C74:G74"/>
+    <mergeCell ref="C75:G75"/>
+    <mergeCell ref="C76:G76"/>
+    <mergeCell ref="C77:G77"/>
+    <mergeCell ref="C78:G78"/>
+    <mergeCell ref="C79:G79"/>
+    <mergeCell ref="C80:G80"/>
+    <mergeCell ref="A35:A44"/>
+    <mergeCell ref="C44:G44"/>
+    <mergeCell ref="A14:A19"/>
+    <mergeCell ref="C39:G39"/>
+    <mergeCell ref="A20:A34"/>
+    <mergeCell ref="B23:B34"/>
+    <mergeCell ref="C24:G24"/>
+    <mergeCell ref="A54:A63"/>
+    <mergeCell ref="B55:B63"/>
+    <mergeCell ref="C55:G55"/>
+    <mergeCell ref="C56:G56"/>
+    <mergeCell ref="C57:G57"/>
+    <mergeCell ref="C58:G58"/>
+    <mergeCell ref="C59:G59"/>
+    <mergeCell ref="C60:G60"/>
+    <mergeCell ref="C61:G61"/>
+    <mergeCell ref="C62:G62"/>
+    <mergeCell ref="C63:G63"/>
+    <mergeCell ref="C54:G54"/>
+    <mergeCell ref="A52:A53"/>
+    <mergeCell ref="C46:G46"/>
+    <mergeCell ref="C45:G45"/>
+    <mergeCell ref="B47:B51"/>
+    <mergeCell ref="A47:A51"/>
+    <mergeCell ref="C47:G47"/>
+    <mergeCell ref="C48:G48"/>
+    <mergeCell ref="C49:G49"/>
+    <mergeCell ref="C50:G50"/>
+    <mergeCell ref="C51:G51"/>
+    <mergeCell ref="C52:G52"/>
+    <mergeCell ref="C53:G53"/>
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="C2:G2"/>
+    <mergeCell ref="A3:A6"/>
+    <mergeCell ref="C3:G3"/>
+    <mergeCell ref="C4:G4"/>
+    <mergeCell ref="C5:G5"/>
+    <mergeCell ref="B4:B6"/>
+    <mergeCell ref="C6:G6"/>
+    <mergeCell ref="C7:G7"/>
+    <mergeCell ref="A7:A13"/>
+    <mergeCell ref="B7:B9"/>
+    <mergeCell ref="B10:B13"/>
+    <mergeCell ref="C8:G8"/>
+    <mergeCell ref="C9:G9"/>
+    <mergeCell ref="C10:G10"/>
+    <mergeCell ref="C11:G11"/>
+    <mergeCell ref="C12:G12"/>
+    <mergeCell ref="C13:G13"/>
+    <mergeCell ref="C41:G41"/>
+    <mergeCell ref="C15:G15"/>
+    <mergeCell ref="C17:G17"/>
+    <mergeCell ref="C19:G19"/>
+    <mergeCell ref="C16:G16"/>
+    <mergeCell ref="B35:B37"/>
+    <mergeCell ref="C35:G35"/>
+    <mergeCell ref="C36:G36"/>
+    <mergeCell ref="C37:G37"/>
+    <mergeCell ref="B18:B19"/>
+    <mergeCell ref="C18:G18"/>
+    <mergeCell ref="B14:B17"/>
     <mergeCell ref="A108:A109"/>
     <mergeCell ref="B108:B109"/>
     <mergeCell ref="C108:G108"/>
@@ -2887,129 +3010,6 @@
     <mergeCell ref="C26:G26"/>
     <mergeCell ref="C22:G22"/>
     <mergeCell ref="C40:G40"/>
-    <mergeCell ref="C13:G13"/>
-    <mergeCell ref="C41:G41"/>
-    <mergeCell ref="C15:G15"/>
-    <mergeCell ref="C17:G17"/>
-    <mergeCell ref="C19:G19"/>
-    <mergeCell ref="C16:G16"/>
-    <mergeCell ref="B35:B37"/>
-    <mergeCell ref="C35:G35"/>
-    <mergeCell ref="C36:G36"/>
-    <mergeCell ref="C37:G37"/>
-    <mergeCell ref="B18:B19"/>
-    <mergeCell ref="C18:G18"/>
-    <mergeCell ref="B14:B17"/>
-    <mergeCell ref="C47:G47"/>
-    <mergeCell ref="C48:G48"/>
-    <mergeCell ref="C49:G49"/>
-    <mergeCell ref="C50:G50"/>
-    <mergeCell ref="C51:G51"/>
-    <mergeCell ref="C52:G52"/>
-    <mergeCell ref="C53:G53"/>
-    <mergeCell ref="A1:G1"/>
-    <mergeCell ref="C2:G2"/>
-    <mergeCell ref="A3:A6"/>
-    <mergeCell ref="C3:G3"/>
-    <mergeCell ref="C4:G4"/>
-    <mergeCell ref="C5:G5"/>
-    <mergeCell ref="B4:B6"/>
-    <mergeCell ref="C6:G6"/>
-    <mergeCell ref="C7:G7"/>
-    <mergeCell ref="A7:A13"/>
-    <mergeCell ref="B7:B9"/>
-    <mergeCell ref="B10:B13"/>
-    <mergeCell ref="C8:G8"/>
-    <mergeCell ref="C9:G9"/>
-    <mergeCell ref="C10:G10"/>
-    <mergeCell ref="C11:G11"/>
-    <mergeCell ref="C12:G12"/>
-    <mergeCell ref="A35:A44"/>
-    <mergeCell ref="C44:G44"/>
-    <mergeCell ref="A14:A19"/>
-    <mergeCell ref="C39:G39"/>
-    <mergeCell ref="A20:A34"/>
-    <mergeCell ref="B23:B34"/>
-    <mergeCell ref="C24:G24"/>
-    <mergeCell ref="A54:A63"/>
-    <mergeCell ref="B55:B63"/>
-    <mergeCell ref="C55:G55"/>
-    <mergeCell ref="C56:G56"/>
-    <mergeCell ref="C57:G57"/>
-    <mergeCell ref="C58:G58"/>
-    <mergeCell ref="C59:G59"/>
-    <mergeCell ref="C60:G60"/>
-    <mergeCell ref="C61:G61"/>
-    <mergeCell ref="C62:G62"/>
-    <mergeCell ref="C63:G63"/>
-    <mergeCell ref="C54:G54"/>
-    <mergeCell ref="A52:A53"/>
-    <mergeCell ref="C46:G46"/>
-    <mergeCell ref="C45:G45"/>
-    <mergeCell ref="B47:B51"/>
-    <mergeCell ref="A47:A51"/>
-    <mergeCell ref="C81:G81"/>
-    <mergeCell ref="B70:B80"/>
-    <mergeCell ref="A70:A80"/>
-    <mergeCell ref="C70:G70"/>
-    <mergeCell ref="C71:G71"/>
-    <mergeCell ref="C72:G72"/>
-    <mergeCell ref="C73:G73"/>
-    <mergeCell ref="C74:G74"/>
-    <mergeCell ref="C75:G75"/>
-    <mergeCell ref="C76:G76"/>
-    <mergeCell ref="C77:G77"/>
-    <mergeCell ref="C78:G78"/>
-    <mergeCell ref="C79:G79"/>
-    <mergeCell ref="C80:G80"/>
-    <mergeCell ref="C68:G68"/>
-    <mergeCell ref="C69:G69"/>
-    <mergeCell ref="A68:A69"/>
-    <mergeCell ref="B68:B69"/>
-    <mergeCell ref="A64:A66"/>
-    <mergeCell ref="C65:G65"/>
-    <mergeCell ref="C66:G66"/>
-    <mergeCell ref="B65:B66"/>
-    <mergeCell ref="C67:G67"/>
-    <mergeCell ref="C64:G64"/>
-    <mergeCell ref="A82:A90"/>
-    <mergeCell ref="B82:B84"/>
-    <mergeCell ref="C89:G89"/>
-    <mergeCell ref="C82:G82"/>
-    <mergeCell ref="C83:G83"/>
-    <mergeCell ref="C84:G84"/>
-    <mergeCell ref="C85:G85"/>
-    <mergeCell ref="C86:G86"/>
-    <mergeCell ref="C87:G87"/>
-    <mergeCell ref="C88:G88"/>
-    <mergeCell ref="C90:G90"/>
-    <mergeCell ref="B85:B90"/>
-    <mergeCell ref="B93:B98"/>
-    <mergeCell ref="A93:A98"/>
-    <mergeCell ref="C93:G93"/>
-    <mergeCell ref="C94:G94"/>
-    <mergeCell ref="C95:G95"/>
-    <mergeCell ref="C96:G96"/>
-    <mergeCell ref="C97:G97"/>
-    <mergeCell ref="C98:G98"/>
-    <mergeCell ref="C91:G91"/>
-    <mergeCell ref="C92:G92"/>
-    <mergeCell ref="B91:B92"/>
-    <mergeCell ref="A91:A92"/>
-    <mergeCell ref="A103:A107"/>
-    <mergeCell ref="B103:B107"/>
-    <mergeCell ref="C103:G103"/>
-    <mergeCell ref="C104:G104"/>
-    <mergeCell ref="C105:G105"/>
-    <mergeCell ref="C106:G106"/>
-    <mergeCell ref="C107:G107"/>
-    <mergeCell ref="A99:A100"/>
-    <mergeCell ref="B99:B100"/>
-    <mergeCell ref="C99:G99"/>
-    <mergeCell ref="C100:G100"/>
-    <mergeCell ref="C101:G101"/>
-    <mergeCell ref="C102:G102"/>
-    <mergeCell ref="A101:A102"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -3027,15 +3027,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A1" s="87">
+      <c r="A1" s="78">
         <v>46235</v>
       </c>
-      <c r="B1" s="87"/>
-      <c r="C1" s="87"/>
-      <c r="D1" s="87"/>
-      <c r="E1" s="87"/>
-      <c r="F1" s="87"/>
-      <c r="G1" s="87"/>
+      <c r="B1" s="78"/>
+      <c r="C1" s="78"/>
+      <c r="D1" s="78"/>
+      <c r="E1" s="78"/>
+      <c r="F1" s="78"/>
+      <c r="G1" s="78"/>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
@@ -3968,7 +3968,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{35F794F4-B843-4D59-B697-A1CBEF2779DC}">
-  <dimension ref="A1:G44"/>
+  <dimension ref="A1:G47"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.140625" style="10"/>
@@ -4372,9 +4372,6 @@
       <c r="C38" s="25" t="s">
         <v>168</v>
       </c>
-      <c r="D38" s="93"/>
-      <c r="E38" s="93"/>
-      <c r="F38" s="93"/>
       <c r="G38" s="51"/>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.25">
@@ -4428,9 +4425,6 @@
       <c r="C42" s="25" t="s">
         <v>171</v>
       </c>
-      <c r="D42" s="93"/>
-      <c r="E42" s="93"/>
-      <c r="F42" s="93"/>
       <c r="G42" s="51"/>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.25">
@@ -4439,9 +4433,6 @@
       <c r="C43" s="25" t="s">
         <v>172</v>
       </c>
-      <c r="D43" s="93"/>
-      <c r="E43" s="93"/>
-      <c r="F43" s="93"/>
       <c r="G43" s="51"/>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.25">
@@ -4454,6 +4445,43 @@
       <c r="E44" s="49"/>
       <c r="F44" s="49"/>
       <c r="G44" s="50"/>
+    </row>
+    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A45" s="11">
+        <v>46284</v>
+      </c>
+      <c r="B45" s="44" t="s">
+        <v>4</v>
+      </c>
+      <c r="C45" s="24" t="s">
+        <v>107</v>
+      </c>
+      <c r="D45" s="47"/>
+      <c r="E45" s="47"/>
+      <c r="F45" s="47"/>
+      <c r="G45" s="48"/>
+    </row>
+    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A46" s="46"/>
+      <c r="B46" s="46"/>
+      <c r="C46" s="25" t="s">
+        <v>71</v>
+      </c>
+      <c r="D46" s="93"/>
+      <c r="E46" s="93"/>
+      <c r="F46" s="93"/>
+      <c r="G46" s="51"/>
+    </row>
+    <row r="47" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A47" s="45"/>
+      <c r="B47" s="45"/>
+      <c r="C47" s="26" t="s">
+        <v>150</v>
+      </c>
+      <c r="D47" s="49"/>
+      <c r="E47" s="49"/>
+      <c r="F47" s="49"/>
+      <c r="G47" s="50"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
Trả BH: SEA, Victory, Ngọc Hoàn
</commit_message>
<xml_diff>
--- a/5. Other/Nội dung công việc hàng ngày.xlsx
+++ b/5. Other/Nội dung công việc hàng ngày.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\VNET\5. Other\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C0EDE018-09B5-43C4-85E2-8D7288DCF56F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AEA41205-1F69-4F52-8030-B5EADD0EDC44}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="3" xr2:uid="{F20CEA29-D7AE-4CD4-9104-84E191A61AC3}"/>
   </bookViews>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="343" uniqueCount="175">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="346" uniqueCount="176">
   <si>
     <t>Hoàn thiện 73 dây nguồn VNSH03</t>
   </si>
@@ -556,6 +556,9 @@
   </si>
   <si>
     <t>Nhận BH Anh Tuấn NB</t>
+  </si>
+  <si>
+    <t>Nhận BH Nguyễn Nam</t>
   </si>
 </sst>
 </file>
@@ -935,6 +938,24 @@
     <xf numFmtId="14" fontId="1" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="17" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -947,9 +968,6 @@
     <xf numFmtId="14" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -959,20 +977,14 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="17" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -980,6 +992,24 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -989,9 +1019,6 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="14" fontId="1" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1001,34 +1028,10 @@
     <xf numFmtId="14" fontId="1" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="17" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1353,15 +1356,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A1" s="71">
+      <c r="A1" s="63">
         <v>46174</v>
       </c>
-      <c r="B1" s="72"/>
-      <c r="C1" s="72"/>
-      <c r="D1" s="72"/>
-      <c r="E1" s="72"/>
-      <c r="F1" s="72"/>
-      <c r="G1" s="72"/>
+      <c r="B1" s="64"/>
+      <c r="C1" s="64"/>
+      <c r="D1" s="64"/>
+      <c r="E1" s="64"/>
+      <c r="F1" s="64"/>
+      <c r="G1" s="64"/>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
@@ -1370,146 +1373,146 @@
       <c r="B2" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C2" s="73" t="s">
+      <c r="C2" s="65" t="s">
         <v>8</v>
       </c>
-      <c r="D2" s="74"/>
-      <c r="E2" s="74"/>
-      <c r="F2" s="74"/>
-      <c r="G2" s="75"/>
+      <c r="D2" s="66"/>
+      <c r="E2" s="66"/>
+      <c r="F2" s="66"/>
+      <c r="G2" s="67"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3" s="66">
+      <c r="A3" s="72">
         <v>46202</v>
       </c>
-      <c r="B3" s="67" t="s">
+      <c r="B3" s="68" t="s">
         <v>5</v>
       </c>
-      <c r="C3" s="67" t="s">
+      <c r="C3" s="68" t="s">
         <v>2</v>
       </c>
-      <c r="D3" s="67"/>
-      <c r="E3" s="67"/>
-      <c r="F3" s="67"/>
-      <c r="G3" s="67"/>
+      <c r="D3" s="68"/>
+      <c r="E3" s="68"/>
+      <c r="F3" s="68"/>
+      <c r="G3" s="68"/>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4" s="66"/>
-      <c r="B4" s="67"/>
-      <c r="C4" s="67" t="s">
+      <c r="A4" s="72"/>
+      <c r="B4" s="68"/>
+      <c r="C4" s="68" t="s">
         <v>0</v>
       </c>
-      <c r="D4" s="67"/>
-      <c r="E4" s="67"/>
-      <c r="F4" s="67"/>
-      <c r="G4" s="67"/>
+      <c r="D4" s="68"/>
+      <c r="E4" s="68"/>
+      <c r="F4" s="68"/>
+      <c r="G4" s="68"/>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" s="66"/>
-      <c r="B5" s="67"/>
-      <c r="C5" s="67" t="s">
+      <c r="A5" s="72"/>
+      <c r="B5" s="68"/>
+      <c r="C5" s="68" t="s">
         <v>3</v>
       </c>
-      <c r="D5" s="67"/>
-      <c r="E5" s="67"/>
-      <c r="F5" s="67"/>
-      <c r="G5" s="67"/>
+      <c r="D5" s="68"/>
+      <c r="E5" s="68"/>
+      <c r="F5" s="68"/>
+      <c r="G5" s="68"/>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" s="66"/>
-      <c r="B6" s="67" t="s">
-        <v>4</v>
-      </c>
-      <c r="C6" s="67" t="s">
+      <c r="A6" s="72"/>
+      <c r="B6" s="68" t="s">
+        <v>4</v>
+      </c>
+      <c r="C6" s="68" t="s">
         <v>1</v>
       </c>
-      <c r="D6" s="67"/>
-      <c r="E6" s="67"/>
-      <c r="F6" s="67"/>
-      <c r="G6" s="67"/>
+      <c r="D6" s="68"/>
+      <c r="E6" s="68"/>
+      <c r="F6" s="68"/>
+      <c r="G6" s="68"/>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A7" s="66"/>
-      <c r="B7" s="67"/>
-      <c r="C7" s="67" t="s">
+      <c r="A7" s="72"/>
+      <c r="B7" s="68"/>
+      <c r="C7" s="68" t="s">
         <v>10</v>
       </c>
-      <c r="D7" s="67"/>
-      <c r="E7" s="67"/>
-      <c r="F7" s="67"/>
-      <c r="G7" s="67"/>
+      <c r="D7" s="68"/>
+      <c r="E7" s="68"/>
+      <c r="F7" s="68"/>
+      <c r="G7" s="68"/>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A8" s="66"/>
-      <c r="B8" s="67"/>
-      <c r="C8" s="67" t="s">
+      <c r="A8" s="72"/>
+      <c r="B8" s="68"/>
+      <c r="C8" s="68" t="s">
         <v>9</v>
       </c>
-      <c r="D8" s="67"/>
-      <c r="E8" s="67"/>
-      <c r="F8" s="67"/>
-      <c r="G8" s="67"/>
+      <c r="D8" s="68"/>
+      <c r="E8" s="68"/>
+      <c r="F8" s="68"/>
+      <c r="G8" s="68"/>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A9" s="66">
+      <c r="A9" s="72">
         <v>46203</v>
       </c>
-      <c r="B9" s="67" t="s">
+      <c r="B9" s="68" t="s">
         <v>5</v>
       </c>
-      <c r="C9" s="68" t="s">
+      <c r="C9" s="73" t="s">
         <v>11</v>
       </c>
-      <c r="D9" s="69"/>
-      <c r="E9" s="69"/>
-      <c r="F9" s="69"/>
-      <c r="G9" s="70"/>
+      <c r="D9" s="74"/>
+      <c r="E9" s="74"/>
+      <c r="F9" s="74"/>
+      <c r="G9" s="75"/>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A10" s="66"/>
-      <c r="B10" s="67"/>
-      <c r="C10" s="63" t="s">
+      <c r="A10" s="72"/>
+      <c r="B10" s="68"/>
+      <c r="C10" s="69" t="s">
         <v>12</v>
       </c>
-      <c r="D10" s="64"/>
-      <c r="E10" s="64"/>
-      <c r="F10" s="64"/>
-      <c r="G10" s="65"/>
+      <c r="D10" s="70"/>
+      <c r="E10" s="70"/>
+      <c r="F10" s="70"/>
+      <c r="G10" s="71"/>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A11" s="66"/>
-      <c r="B11" s="67"/>
-      <c r="C11" s="63" t="s">
+      <c r="A11" s="72"/>
+      <c r="B11" s="68"/>
+      <c r="C11" s="69" t="s">
         <v>13</v>
       </c>
-      <c r="D11" s="64"/>
-      <c r="E11" s="64"/>
-      <c r="F11" s="64"/>
-      <c r="G11" s="65"/>
+      <c r="D11" s="70"/>
+      <c r="E11" s="70"/>
+      <c r="F11" s="70"/>
+      <c r="G11" s="71"/>
     </row>
     <row r="12" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="66"/>
-      <c r="B12" s="67"/>
-      <c r="C12" s="63" t="s">
+      <c r="A12" s="72"/>
+      <c r="B12" s="68"/>
+      <c r="C12" s="69" t="s">
         <v>14</v>
       </c>
-      <c r="D12" s="64"/>
-      <c r="E12" s="64"/>
-      <c r="F12" s="64"/>
-      <c r="G12" s="65"/>
+      <c r="D12" s="70"/>
+      <c r="E12" s="70"/>
+      <c r="F12" s="70"/>
+      <c r="G12" s="71"/>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A13" s="66"/>
+      <c r="A13" s="72"/>
       <c r="B13" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="C13" s="63" t="s">
+      <c r="C13" s="69" t="s">
         <v>9</v>
       </c>
-      <c r="D13" s="64"/>
-      <c r="E13" s="64"/>
-      <c r="F13" s="64"/>
-      <c r="G13" s="65"/>
+      <c r="D13" s="70"/>
+      <c r="E13" s="70"/>
+      <c r="F13" s="70"/>
+      <c r="G13" s="71"/>
     </row>
   </sheetData>
   <autoFilter ref="A2:G8" xr:uid="{5B424F82-FB95-405B-80D1-35D47957B3B0}">
@@ -1519,6 +1522,14 @@
     <filterColumn colId="5" showButton="0"/>
   </autoFilter>
   <mergeCells count="18">
+    <mergeCell ref="C12:G12"/>
+    <mergeCell ref="C13:G13"/>
+    <mergeCell ref="A9:A13"/>
+    <mergeCell ref="B9:B12"/>
+    <mergeCell ref="A3:A8"/>
+    <mergeCell ref="C9:G9"/>
+    <mergeCell ref="C10:G10"/>
+    <mergeCell ref="C11:G11"/>
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="C2:G2"/>
     <mergeCell ref="B6:B8"/>
@@ -1529,14 +1540,6 @@
     <mergeCell ref="C5:G5"/>
     <mergeCell ref="C6:G6"/>
     <mergeCell ref="C7:G7"/>
-    <mergeCell ref="C12:G12"/>
-    <mergeCell ref="C13:G13"/>
-    <mergeCell ref="A9:A13"/>
-    <mergeCell ref="B9:B12"/>
-    <mergeCell ref="A3:A8"/>
-    <mergeCell ref="C9:G9"/>
-    <mergeCell ref="C10:G10"/>
-    <mergeCell ref="C11:G11"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1554,15 +1557,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A1" s="79">
+      <c r="A1" s="88">
         <v>46204</v>
       </c>
-      <c r="B1" s="79"/>
-      <c r="C1" s="79"/>
-      <c r="D1" s="79"/>
-      <c r="E1" s="79"/>
-      <c r="F1" s="79"/>
-      <c r="G1" s="79"/>
+      <c r="B1" s="88"/>
+      <c r="C1" s="88"/>
+      <c r="D1" s="88"/>
+      <c r="E1" s="88"/>
+      <c r="F1" s="88"/>
+      <c r="G1" s="88"/>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
@@ -1571,152 +1574,152 @@
       <c r="B2" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C2" s="80" t="s">
+      <c r="C2" s="89" t="s">
         <v>8</v>
       </c>
-      <c r="D2" s="80"/>
-      <c r="E2" s="80"/>
-      <c r="F2" s="80"/>
-      <c r="G2" s="80"/>
+      <c r="D2" s="89"/>
+      <c r="E2" s="89"/>
+      <c r="F2" s="89"/>
+      <c r="G2" s="89"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3" s="66">
+      <c r="A3" s="72">
         <v>46204</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="C3" s="67" t="s">
+      <c r="C3" s="68" t="s">
         <v>15</v>
       </c>
-      <c r="D3" s="67"/>
-      <c r="E3" s="67"/>
-      <c r="F3" s="67"/>
-      <c r="G3" s="67"/>
+      <c r="D3" s="68"/>
+      <c r="E3" s="68"/>
+      <c r="F3" s="68"/>
+      <c r="G3" s="68"/>
     </row>
     <row r="4" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="66"/>
-      <c r="B4" s="67" t="s">
-        <v>4</v>
-      </c>
-      <c r="C4" s="81" t="s">
+      <c r="A4" s="72"/>
+      <c r="B4" s="68" t="s">
+        <v>4</v>
+      </c>
+      <c r="C4" s="77" t="s">
         <v>16</v>
       </c>
-      <c r="D4" s="81"/>
-      <c r="E4" s="81"/>
-      <c r="F4" s="81"/>
-      <c r="G4" s="81"/>
+      <c r="D4" s="77"/>
+      <c r="E4" s="77"/>
+      <c r="F4" s="77"/>
+      <c r="G4" s="77"/>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" s="66"/>
-      <c r="B5" s="67"/>
-      <c r="C5" s="67" t="s">
+      <c r="A5" s="72"/>
+      <c r="B5" s="68"/>
+      <c r="C5" s="68" t="s">
         <v>17</v>
       </c>
-      <c r="D5" s="67"/>
-      <c r="E5" s="67"/>
-      <c r="F5" s="67"/>
-      <c r="G5" s="67"/>
+      <c r="D5" s="68"/>
+      <c r="E5" s="68"/>
+      <c r="F5" s="68"/>
+      <c r="G5" s="68"/>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" s="66"/>
-      <c r="B6" s="67"/>
-      <c r="C6" s="67" t="s">
+      <c r="A6" s="72"/>
+      <c r="B6" s="68"/>
+      <c r="C6" s="68" t="s">
         <v>18</v>
       </c>
-      <c r="D6" s="67"/>
-      <c r="E6" s="67"/>
-      <c r="F6" s="67"/>
-      <c r="G6" s="67"/>
+      <c r="D6" s="68"/>
+      <c r="E6" s="68"/>
+      <c r="F6" s="68"/>
+      <c r="G6" s="68"/>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A7" s="82">
+      <c r="A7" s="90">
         <v>46205</v>
       </c>
-      <c r="B7" s="76" t="s">
+      <c r="B7" s="79" t="s">
         <v>5</v>
       </c>
-      <c r="C7" s="68" t="s">
+      <c r="C7" s="73" t="s">
         <v>25</v>
       </c>
-      <c r="D7" s="69"/>
-      <c r="E7" s="69"/>
-      <c r="F7" s="69"/>
-      <c r="G7" s="70"/>
+      <c r="D7" s="74"/>
+      <c r="E7" s="74"/>
+      <c r="F7" s="74"/>
+      <c r="G7" s="75"/>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A8" s="83"/>
-      <c r="B8" s="78"/>
-      <c r="C8" s="63" t="s">
+      <c r="A8" s="91"/>
+      <c r="B8" s="87"/>
+      <c r="C8" s="69" t="s">
         <v>19</v>
       </c>
-      <c r="D8" s="64"/>
-      <c r="E8" s="64"/>
-      <c r="F8" s="64"/>
-      <c r="G8" s="65"/>
+      <c r="D8" s="70"/>
+      <c r="E8" s="70"/>
+      <c r="F8" s="70"/>
+      <c r="G8" s="71"/>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A9" s="83"/>
-      <c r="B9" s="77"/>
-      <c r="C9" s="63" t="s">
+      <c r="A9" s="91"/>
+      <c r="B9" s="80"/>
+      <c r="C9" s="69" t="s">
         <v>24</v>
       </c>
-      <c r="D9" s="64"/>
-      <c r="E9" s="64"/>
-      <c r="F9" s="64"/>
-      <c r="G9" s="65"/>
+      <c r="D9" s="70"/>
+      <c r="E9" s="70"/>
+      <c r="F9" s="70"/>
+      <c r="G9" s="71"/>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A10" s="83"/>
-      <c r="B10" s="67" t="s">
-        <v>4</v>
-      </c>
-      <c r="C10" s="63" t="s">
+      <c r="A10" s="91"/>
+      <c r="B10" s="68" t="s">
+        <v>4</v>
+      </c>
+      <c r="C10" s="69" t="s">
         <v>22</v>
       </c>
-      <c r="D10" s="64"/>
-      <c r="E10" s="64"/>
-      <c r="F10" s="64"/>
-      <c r="G10" s="65"/>
+      <c r="D10" s="70"/>
+      <c r="E10" s="70"/>
+      <c r="F10" s="70"/>
+      <c r="G10" s="71"/>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A11" s="83"/>
-      <c r="B11" s="67"/>
-      <c r="C11" s="63" t="s">
+      <c r="A11" s="91"/>
+      <c r="B11" s="68"/>
+      <c r="C11" s="69" t="s">
         <v>20</v>
       </c>
-      <c r="D11" s="64"/>
-      <c r="E11" s="64"/>
-      <c r="F11" s="64"/>
-      <c r="G11" s="65"/>
+      <c r="D11" s="70"/>
+      <c r="E11" s="70"/>
+      <c r="F11" s="70"/>
+      <c r="G11" s="71"/>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A12" s="83"/>
-      <c r="B12" s="67"/>
-      <c r="C12" s="63" t="s">
+      <c r="A12" s="91"/>
+      <c r="B12" s="68"/>
+      <c r="C12" s="69" t="s">
         <v>21</v>
       </c>
-      <c r="D12" s="64"/>
-      <c r="E12" s="64"/>
-      <c r="F12" s="64"/>
-      <c r="G12" s="65"/>
+      <c r="D12" s="70"/>
+      <c r="E12" s="70"/>
+      <c r="F12" s="70"/>
+      <c r="G12" s="71"/>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A13" s="84"/>
-      <c r="B13" s="67"/>
-      <c r="C13" s="63" t="s">
+      <c r="A13" s="92"/>
+      <c r="B13" s="68"/>
+      <c r="C13" s="69" t="s">
         <v>23</v>
       </c>
-      <c r="D13" s="64"/>
-      <c r="E13" s="64"/>
-      <c r="F13" s="64"/>
-      <c r="G13" s="65"/>
+      <c r="D13" s="70"/>
+      <c r="E13" s="70"/>
+      <c r="F13" s="70"/>
+      <c r="G13" s="71"/>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A14" s="86">
+      <c r="A14" s="81">
         <v>46206</v>
       </c>
-      <c r="B14" s="76" t="s">
+      <c r="B14" s="79" t="s">
         <v>5</v>
       </c>
       <c r="C14" s="3" t="s">
@@ -1728,348 +1731,348 @@
       <c r="G14" s="5"/>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A15" s="87"/>
-      <c r="B15" s="78"/>
-      <c r="C15" s="68" t="s">
+      <c r="A15" s="84"/>
+      <c r="B15" s="87"/>
+      <c r="C15" s="73" t="s">
         <v>26</v>
       </c>
-      <c r="D15" s="69"/>
-      <c r="E15" s="69"/>
-      <c r="F15" s="69"/>
-      <c r="G15" s="70"/>
+      <c r="D15" s="74"/>
+      <c r="E15" s="74"/>
+      <c r="F15" s="74"/>
+      <c r="G15" s="75"/>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A16" s="87"/>
-      <c r="B16" s="78"/>
-      <c r="C16" s="68" t="s">
+      <c r="A16" s="84"/>
+      <c r="B16" s="87"/>
+      <c r="C16" s="73" t="s">
         <v>28</v>
       </c>
-      <c r="D16" s="69"/>
-      <c r="E16" s="69"/>
-      <c r="F16" s="69"/>
-      <c r="G16" s="70"/>
+      <c r="D16" s="74"/>
+      <c r="E16" s="74"/>
+      <c r="F16" s="74"/>
+      <c r="G16" s="75"/>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A17" s="87"/>
-      <c r="B17" s="77"/>
-      <c r="C17" s="68" t="s">
+      <c r="A17" s="84"/>
+      <c r="B17" s="80"/>
+      <c r="C17" s="73" t="s">
         <v>27</v>
       </c>
-      <c r="D17" s="69"/>
-      <c r="E17" s="69"/>
-      <c r="F17" s="69"/>
-      <c r="G17" s="70"/>
+      <c r="D17" s="74"/>
+      <c r="E17" s="74"/>
+      <c r="F17" s="74"/>
+      <c r="G17" s="75"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A18" s="87"/>
-      <c r="B18" s="76" t="s">
-        <v>4</v>
-      </c>
-      <c r="C18" s="68" t="s">
+      <c r="A18" s="84"/>
+      <c r="B18" s="79" t="s">
+        <v>4</v>
+      </c>
+      <c r="C18" s="73" t="s">
         <v>29</v>
       </c>
-      <c r="D18" s="69"/>
-      <c r="E18" s="69"/>
-      <c r="F18" s="69"/>
-      <c r="G18" s="70"/>
+      <c r="D18" s="74"/>
+      <c r="E18" s="74"/>
+      <c r="F18" s="74"/>
+      <c r="G18" s="75"/>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A19" s="88"/>
-      <c r="B19" s="77"/>
-      <c r="C19" s="68" t="s">
+      <c r="A19" s="82"/>
+      <c r="B19" s="80"/>
+      <c r="C19" s="73" t="s">
         <v>31</v>
       </c>
-      <c r="D19" s="69"/>
-      <c r="E19" s="69"/>
-      <c r="F19" s="69"/>
-      <c r="G19" s="70"/>
+      <c r="D19" s="74"/>
+      <c r="E19" s="74"/>
+      <c r="F19" s="74"/>
+      <c r="G19" s="75"/>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A20" s="89">
+      <c r="A20" s="85">
         <v>46209</v>
       </c>
-      <c r="B20" s="67" t="s">
+      <c r="B20" s="68" t="s">
         <v>5</v>
       </c>
-      <c r="C20" s="67" t="s">
+      <c r="C20" s="68" t="s">
         <v>33</v>
       </c>
-      <c r="D20" s="67"/>
-      <c r="E20" s="67"/>
-      <c r="F20" s="67"/>
-      <c r="G20" s="67"/>
+      <c r="D20" s="68"/>
+      <c r="E20" s="68"/>
+      <c r="F20" s="68"/>
+      <c r="G20" s="68"/>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A21" s="89"/>
-      <c r="B21" s="67"/>
-      <c r="C21" s="67" t="s">
+      <c r="A21" s="85"/>
+      <c r="B21" s="68"/>
+      <c r="C21" s="68" t="s">
         <v>34</v>
       </c>
-      <c r="D21" s="67"/>
-      <c r="E21" s="67"/>
-      <c r="F21" s="67"/>
-      <c r="G21" s="67"/>
+      <c r="D21" s="68"/>
+      <c r="E21" s="68"/>
+      <c r="F21" s="68"/>
+      <c r="G21" s="68"/>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A22" s="89"/>
-      <c r="B22" s="67"/>
-      <c r="C22" s="67" t="s">
+      <c r="A22" s="85"/>
+      <c r="B22" s="68"/>
+      <c r="C22" s="68" t="s">
         <v>15</v>
       </c>
-      <c r="D22" s="67"/>
-      <c r="E22" s="67"/>
-      <c r="F22" s="67"/>
-      <c r="G22" s="67"/>
+      <c r="D22" s="68"/>
+      <c r="E22" s="68"/>
+      <c r="F22" s="68"/>
+      <c r="G22" s="68"/>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A23" s="89"/>
-      <c r="B23" s="67" t="s">
-        <v>4</v>
-      </c>
-      <c r="C23" s="67" t="s">
+      <c r="A23" s="85"/>
+      <c r="B23" s="68" t="s">
+        <v>4</v>
+      </c>
+      <c r="C23" s="68" t="s">
         <v>32</v>
       </c>
-      <c r="D23" s="67"/>
-      <c r="E23" s="67"/>
-      <c r="F23" s="67"/>
-      <c r="G23" s="67"/>
+      <c r="D23" s="68"/>
+      <c r="E23" s="68"/>
+      <c r="F23" s="68"/>
+      <c r="G23" s="68"/>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A24" s="89"/>
-      <c r="B24" s="67"/>
-      <c r="C24" s="68" t="s">
+      <c r="A24" s="85"/>
+      <c r="B24" s="68"/>
+      <c r="C24" s="73" t="s">
         <v>35</v>
       </c>
-      <c r="D24" s="69"/>
-      <c r="E24" s="69"/>
-      <c r="F24" s="69"/>
-      <c r="G24" s="70"/>
+      <c r="D24" s="74"/>
+      <c r="E24" s="74"/>
+      <c r="F24" s="74"/>
+      <c r="G24" s="75"/>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A25" s="89"/>
-      <c r="B25" s="67"/>
-      <c r="C25" s="68" t="s">
+      <c r="A25" s="85"/>
+      <c r="B25" s="68"/>
+      <c r="C25" s="73" t="s">
         <v>36</v>
       </c>
-      <c r="D25" s="69"/>
-      <c r="E25" s="69"/>
-      <c r="F25" s="69"/>
-      <c r="G25" s="70"/>
+      <c r="D25" s="74"/>
+      <c r="E25" s="74"/>
+      <c r="F25" s="74"/>
+      <c r="G25" s="75"/>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A26" s="89"/>
-      <c r="B26" s="67"/>
-      <c r="C26" s="68" t="s">
+      <c r="A26" s="85"/>
+      <c r="B26" s="68"/>
+      <c r="C26" s="73" t="s">
         <v>37</v>
       </c>
-      <c r="D26" s="69"/>
-      <c r="E26" s="69"/>
-      <c r="F26" s="69"/>
-      <c r="G26" s="70"/>
+      <c r="D26" s="74"/>
+      <c r="E26" s="74"/>
+      <c r="F26" s="74"/>
+      <c r="G26" s="75"/>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A27" s="89"/>
-      <c r="B27" s="67"/>
-      <c r="C27" s="68" t="s">
+      <c r="A27" s="85"/>
+      <c r="B27" s="68"/>
+      <c r="C27" s="73" t="s">
         <v>38</v>
       </c>
-      <c r="D27" s="69"/>
-      <c r="E27" s="69"/>
-      <c r="F27" s="69"/>
-      <c r="G27" s="70"/>
+      <c r="D27" s="74"/>
+      <c r="E27" s="74"/>
+      <c r="F27" s="74"/>
+      <c r="G27" s="75"/>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A28" s="89"/>
-      <c r="B28" s="67"/>
-      <c r="C28" s="68" t="s">
+      <c r="A28" s="85"/>
+      <c r="B28" s="68"/>
+      <c r="C28" s="73" t="s">
         <v>39</v>
       </c>
-      <c r="D28" s="69"/>
-      <c r="E28" s="69"/>
-      <c r="F28" s="69"/>
-      <c r="G28" s="70"/>
+      <c r="D28" s="74"/>
+      <c r="E28" s="74"/>
+      <c r="F28" s="74"/>
+      <c r="G28" s="75"/>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A29" s="89"/>
-      <c r="B29" s="67"/>
-      <c r="C29" s="68" t="s">
+      <c r="A29" s="85"/>
+      <c r="B29" s="68"/>
+      <c r="C29" s="73" t="s">
         <v>40</v>
       </c>
-      <c r="D29" s="69"/>
-      <c r="E29" s="69"/>
-      <c r="F29" s="69"/>
-      <c r="G29" s="70"/>
+      <c r="D29" s="74"/>
+      <c r="E29" s="74"/>
+      <c r="F29" s="74"/>
+      <c r="G29" s="75"/>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A30" s="89"/>
-      <c r="B30" s="67"/>
-      <c r="C30" s="68" t="s">
+      <c r="A30" s="85"/>
+      <c r="B30" s="68"/>
+      <c r="C30" s="73" t="s">
         <v>45</v>
       </c>
-      <c r="D30" s="69"/>
-      <c r="E30" s="69"/>
-      <c r="F30" s="69"/>
-      <c r="G30" s="70"/>
+      <c r="D30" s="74"/>
+      <c r="E30" s="74"/>
+      <c r="F30" s="74"/>
+      <c r="G30" s="75"/>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A31" s="89"/>
-      <c r="B31" s="67"/>
-      <c r="C31" s="68" t="s">
+      <c r="A31" s="85"/>
+      <c r="B31" s="68"/>
+      <c r="C31" s="73" t="s">
         <v>41</v>
       </c>
-      <c r="D31" s="69"/>
-      <c r="E31" s="69"/>
-      <c r="F31" s="69"/>
-      <c r="G31" s="70"/>
+      <c r="D31" s="74"/>
+      <c r="E31" s="74"/>
+      <c r="F31" s="74"/>
+      <c r="G31" s="75"/>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A32" s="89"/>
-      <c r="B32" s="67"/>
-      <c r="C32" s="68" t="s">
+      <c r="A32" s="85"/>
+      <c r="B32" s="68"/>
+      <c r="C32" s="73" t="s">
         <v>42</v>
       </c>
-      <c r="D32" s="69"/>
-      <c r="E32" s="69"/>
-      <c r="F32" s="69"/>
-      <c r="G32" s="70"/>
+      <c r="D32" s="74"/>
+      <c r="E32" s="74"/>
+      <c r="F32" s="74"/>
+      <c r="G32" s="75"/>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A33" s="89"/>
-      <c r="B33" s="67"/>
-      <c r="C33" s="68" t="s">
+      <c r="A33" s="85"/>
+      <c r="B33" s="68"/>
+      <c r="C33" s="73" t="s">
         <v>43</v>
       </c>
-      <c r="D33" s="69"/>
-      <c r="E33" s="69"/>
-      <c r="F33" s="69"/>
-      <c r="G33" s="70"/>
+      <c r="D33" s="74"/>
+      <c r="E33" s="74"/>
+      <c r="F33" s="74"/>
+      <c r="G33" s="75"/>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A34" s="89"/>
-      <c r="B34" s="67"/>
-      <c r="C34" s="68" t="s">
+      <c r="A34" s="85"/>
+      <c r="B34" s="68"/>
+      <c r="C34" s="73" t="s">
         <v>44</v>
       </c>
-      <c r="D34" s="69"/>
-      <c r="E34" s="69"/>
-      <c r="F34" s="69"/>
-      <c r="G34" s="70"/>
+      <c r="D34" s="74"/>
+      <c r="E34" s="74"/>
+      <c r="F34" s="74"/>
+      <c r="G34" s="75"/>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A35" s="85">
+      <c r="A35" s="83">
         <v>46210</v>
       </c>
-      <c r="B35" s="67" t="s">
+      <c r="B35" s="68" t="s">
         <v>5</v>
       </c>
-      <c r="C35" s="67" t="s">
+      <c r="C35" s="68" t="s">
         <v>46</v>
       </c>
-      <c r="D35" s="67"/>
-      <c r="E35" s="67"/>
-      <c r="F35" s="67"/>
-      <c r="G35" s="67"/>
+      <c r="D35" s="68"/>
+      <c r="E35" s="68"/>
+      <c r="F35" s="68"/>
+      <c r="G35" s="68"/>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A36" s="85"/>
-      <c r="B36" s="67"/>
-      <c r="C36" s="67" t="s">
+      <c r="A36" s="83"/>
+      <c r="B36" s="68"/>
+      <c r="C36" s="68" t="s">
         <v>27</v>
       </c>
-      <c r="D36" s="67"/>
-      <c r="E36" s="67"/>
-      <c r="F36" s="67"/>
-      <c r="G36" s="67"/>
+      <c r="D36" s="68"/>
+      <c r="E36" s="68"/>
+      <c r="F36" s="68"/>
+      <c r="G36" s="68"/>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A37" s="85"/>
-      <c r="B37" s="67"/>
-      <c r="C37" s="67" t="s">
+      <c r="A37" s="83"/>
+      <c r="B37" s="68"/>
+      <c r="C37" s="68" t="s">
         <v>47</v>
       </c>
-      <c r="D37" s="67"/>
-      <c r="E37" s="67"/>
-      <c r="F37" s="67"/>
-      <c r="G37" s="67"/>
+      <c r="D37" s="68"/>
+      <c r="E37" s="68"/>
+      <c r="F37" s="68"/>
+      <c r="G37" s="68"/>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A38" s="85"/>
-      <c r="B38" s="67" t="s">
-        <v>4</v>
-      </c>
-      <c r="C38" s="67" t="s">
+      <c r="A38" s="83"/>
+      <c r="B38" s="68" t="s">
+        <v>4</v>
+      </c>
+      <c r="C38" s="68" t="s">
         <v>52</v>
       </c>
-      <c r="D38" s="67"/>
-      <c r="E38" s="67"/>
-      <c r="F38" s="67"/>
-      <c r="G38" s="67"/>
+      <c r="D38" s="68"/>
+      <c r="E38" s="68"/>
+      <c r="F38" s="68"/>
+      <c r="G38" s="68"/>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A39" s="85"/>
-      <c r="B39" s="67"/>
-      <c r="C39" s="67" t="s">
+      <c r="A39" s="83"/>
+      <c r="B39" s="68"/>
+      <c r="C39" s="68" t="s">
         <v>53</v>
       </c>
-      <c r="D39" s="67"/>
-      <c r="E39" s="67"/>
-      <c r="F39" s="67"/>
-      <c r="G39" s="67"/>
+      <c r="D39" s="68"/>
+      <c r="E39" s="68"/>
+      <c r="F39" s="68"/>
+      <c r="G39" s="68"/>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A40" s="85"/>
-      <c r="B40" s="67"/>
-      <c r="C40" s="67" t="s">
+      <c r="A40" s="83"/>
+      <c r="B40" s="68"/>
+      <c r="C40" s="68" t="s">
         <v>48</v>
       </c>
-      <c r="D40" s="67"/>
-      <c r="E40" s="67"/>
-      <c r="F40" s="67"/>
-      <c r="G40" s="67"/>
+      <c r="D40" s="68"/>
+      <c r="E40" s="68"/>
+      <c r="F40" s="68"/>
+      <c r="G40" s="68"/>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A41" s="85"/>
-      <c r="B41" s="67"/>
-      <c r="C41" s="67" t="s">
+      <c r="A41" s="83"/>
+      <c r="B41" s="68"/>
+      <c r="C41" s="68" t="s">
         <v>49</v>
       </c>
-      <c r="D41" s="67"/>
-      <c r="E41" s="67"/>
-      <c r="F41" s="67"/>
-      <c r="G41" s="67"/>
+      <c r="D41" s="68"/>
+      <c r="E41" s="68"/>
+      <c r="F41" s="68"/>
+      <c r="G41" s="68"/>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A42" s="85"/>
-      <c r="B42" s="67"/>
-      <c r="C42" s="67" t="s">
+      <c r="A42" s="83"/>
+      <c r="B42" s="68"/>
+      <c r="C42" s="68" t="s">
         <v>50</v>
       </c>
-      <c r="D42" s="67"/>
-      <c r="E42" s="67"/>
-      <c r="F42" s="67"/>
-      <c r="G42" s="67"/>
+      <c r="D42" s="68"/>
+      <c r="E42" s="68"/>
+      <c r="F42" s="68"/>
+      <c r="G42" s="68"/>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A43" s="85"/>
-      <c r="B43" s="67"/>
-      <c r="C43" s="67" t="s">
+      <c r="A43" s="83"/>
+      <c r="B43" s="68"/>
+      <c r="C43" s="68" t="s">
         <v>51</v>
       </c>
-      <c r="D43" s="67"/>
-      <c r="E43" s="67"/>
-      <c r="F43" s="67"/>
-      <c r="G43" s="67"/>
+      <c r="D43" s="68"/>
+      <c r="E43" s="68"/>
+      <c r="F43" s="68"/>
+      <c r="G43" s="68"/>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A44" s="85"/>
-      <c r="B44" s="67"/>
-      <c r="C44" s="68" t="s">
+      <c r="A44" s="83"/>
+      <c r="B44" s="68"/>
+      <c r="C44" s="73" t="s">
         <v>54</v>
       </c>
-      <c r="D44" s="69"/>
-      <c r="E44" s="69"/>
-      <c r="F44" s="69"/>
-      <c r="G44" s="70"/>
+      <c r="D44" s="74"/>
+      <c r="E44" s="74"/>
+      <c r="F44" s="74"/>
+      <c r="G44" s="75"/>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A45" s="6">
@@ -2078,13 +2081,13 @@
       <c r="B45" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="C45" s="67" t="s">
+      <c r="C45" s="68" t="s">
         <v>55</v>
       </c>
-      <c r="D45" s="67"/>
-      <c r="E45" s="67"/>
-      <c r="F45" s="67"/>
-      <c r="G45" s="67"/>
+      <c r="D45" s="68"/>
+      <c r="E45" s="68"/>
+      <c r="F45" s="68"/>
+      <c r="G45" s="68"/>
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A46" s="6">
@@ -2093,255 +2096,255 @@
       <c r="B46" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="C46" s="67" t="s">
+      <c r="C46" s="68" t="s">
         <v>59</v>
       </c>
-      <c r="D46" s="67"/>
-      <c r="E46" s="67"/>
-      <c r="F46" s="67"/>
-      <c r="G46" s="67"/>
+      <c r="D46" s="68"/>
+      <c r="E46" s="68"/>
+      <c r="F46" s="68"/>
+      <c r="G46" s="68"/>
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A47" s="86">
+      <c r="A47" s="81">
         <v>46213</v>
       </c>
-      <c r="B47" s="76" t="s">
-        <v>4</v>
-      </c>
-      <c r="C47" s="68" t="s">
+      <c r="B47" s="79" t="s">
+        <v>4</v>
+      </c>
+      <c r="C47" s="73" t="s">
         <v>56</v>
       </c>
-      <c r="D47" s="69"/>
-      <c r="E47" s="69"/>
-      <c r="F47" s="69"/>
-      <c r="G47" s="70"/>
+      <c r="D47" s="74"/>
+      <c r="E47" s="74"/>
+      <c r="F47" s="74"/>
+      <c r="G47" s="75"/>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A48" s="87"/>
-      <c r="B48" s="78"/>
-      <c r="C48" s="68" t="s">
+      <c r="A48" s="84"/>
+      <c r="B48" s="87"/>
+      <c r="C48" s="73" t="s">
         <v>57</v>
       </c>
-      <c r="D48" s="69"/>
-      <c r="E48" s="69"/>
-      <c r="F48" s="69"/>
-      <c r="G48" s="70"/>
+      <c r="D48" s="74"/>
+      <c r="E48" s="74"/>
+      <c r="F48" s="74"/>
+      <c r="G48" s="75"/>
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A49" s="87"/>
-      <c r="B49" s="78"/>
-      <c r="C49" s="68" t="s">
+      <c r="A49" s="84"/>
+      <c r="B49" s="87"/>
+      <c r="C49" s="73" t="s">
         <v>58</v>
       </c>
-      <c r="D49" s="69"/>
-      <c r="E49" s="69"/>
-      <c r="F49" s="69"/>
-      <c r="G49" s="70"/>
+      <c r="D49" s="74"/>
+      <c r="E49" s="74"/>
+      <c r="F49" s="74"/>
+      <c r="G49" s="75"/>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A50" s="87"/>
-      <c r="B50" s="78"/>
-      <c r="C50" s="68" t="s">
+      <c r="A50" s="84"/>
+      <c r="B50" s="87"/>
+      <c r="C50" s="73" t="s">
         <v>60</v>
       </c>
-      <c r="D50" s="69"/>
-      <c r="E50" s="69"/>
-      <c r="F50" s="69"/>
-      <c r="G50" s="70"/>
+      <c r="D50" s="74"/>
+      <c r="E50" s="74"/>
+      <c r="F50" s="74"/>
+      <c r="G50" s="75"/>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A51" s="88"/>
-      <c r="B51" s="77"/>
-      <c r="C51" s="68" t="s">
+      <c r="A51" s="82"/>
+      <c r="B51" s="80"/>
+      <c r="C51" s="73" t="s">
         <v>61</v>
       </c>
-      <c r="D51" s="69"/>
-      <c r="E51" s="69"/>
-      <c r="F51" s="69"/>
-      <c r="G51" s="70"/>
+      <c r="D51" s="74"/>
+      <c r="E51" s="74"/>
+      <c r="F51" s="74"/>
+      <c r="G51" s="75"/>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A52" s="66">
+      <c r="A52" s="72">
         <v>46214</v>
       </c>
       <c r="B52" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="C52" s="67" t="s">
+      <c r="C52" s="68" t="s">
         <v>62</v>
       </c>
-      <c r="D52" s="67"/>
-      <c r="E52" s="67"/>
-      <c r="F52" s="67"/>
-      <c r="G52" s="67"/>
+      <c r="D52" s="68"/>
+      <c r="E52" s="68"/>
+      <c r="F52" s="68"/>
+      <c r="G52" s="68"/>
     </row>
     <row r="53" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A53" s="66"/>
+      <c r="A53" s="72"/>
       <c r="B53" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="C53" s="67" t="s">
+      <c r="C53" s="68" t="s">
         <v>63</v>
       </c>
-      <c r="D53" s="67"/>
-      <c r="E53" s="67"/>
-      <c r="F53" s="67"/>
-      <c r="G53" s="67"/>
+      <c r="D53" s="68"/>
+      <c r="E53" s="68"/>
+      <c r="F53" s="68"/>
+      <c r="G53" s="68"/>
     </row>
     <row r="54" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A54" s="66">
+      <c r="A54" s="72">
         <v>46216</v>
       </c>
       <c r="B54" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="C54" s="68" t="s">
+      <c r="C54" s="73" t="s">
         <v>70</v>
       </c>
-      <c r="D54" s="69"/>
-      <c r="E54" s="69"/>
-      <c r="F54" s="69"/>
-      <c r="G54" s="70"/>
+      <c r="D54" s="74"/>
+      <c r="E54" s="74"/>
+      <c r="F54" s="74"/>
+      <c r="G54" s="75"/>
     </row>
     <row r="55" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A55" s="66"/>
-      <c r="B55" s="67" t="s">
-        <v>4</v>
-      </c>
-      <c r="C55" s="90" t="s">
+      <c r="A55" s="72"/>
+      <c r="B55" s="68" t="s">
+        <v>4</v>
+      </c>
+      <c r="C55" s="86" t="s">
         <v>65</v>
       </c>
-      <c r="D55" s="90"/>
-      <c r="E55" s="90"/>
-      <c r="F55" s="90"/>
-      <c r="G55" s="90"/>
+      <c r="D55" s="86"/>
+      <c r="E55" s="86"/>
+      <c r="F55" s="86"/>
+      <c r="G55" s="86"/>
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A56" s="66"/>
-      <c r="B56" s="67"/>
-      <c r="C56" s="90" t="s">
+      <c r="A56" s="72"/>
+      <c r="B56" s="68"/>
+      <c r="C56" s="86" t="s">
         <v>66</v>
       </c>
-      <c r="D56" s="90"/>
-      <c r="E56" s="90"/>
-      <c r="F56" s="90"/>
-      <c r="G56" s="90"/>
+      <c r="D56" s="86"/>
+      <c r="E56" s="86"/>
+      <c r="F56" s="86"/>
+      <c r="G56" s="86"/>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A57" s="66"/>
-      <c r="B57" s="67"/>
-      <c r="C57" s="90" t="s">
+      <c r="A57" s="72"/>
+      <c r="B57" s="68"/>
+      <c r="C57" s="86" t="s">
         <v>67</v>
       </c>
-      <c r="D57" s="90"/>
-      <c r="E57" s="90"/>
-      <c r="F57" s="90"/>
-      <c r="G57" s="90"/>
+      <c r="D57" s="86"/>
+      <c r="E57" s="86"/>
+      <c r="F57" s="86"/>
+      <c r="G57" s="86"/>
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A58" s="66"/>
-      <c r="B58" s="67"/>
-      <c r="C58" s="90" t="s">
+      <c r="A58" s="72"/>
+      <c r="B58" s="68"/>
+      <c r="C58" s="86" t="s">
         <v>68</v>
       </c>
-      <c r="D58" s="90"/>
-      <c r="E58" s="90"/>
-      <c r="F58" s="90"/>
-      <c r="G58" s="90"/>
+      <c r="D58" s="86"/>
+      <c r="E58" s="86"/>
+      <c r="F58" s="86"/>
+      <c r="G58" s="86"/>
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A59" s="66"/>
-      <c r="B59" s="67"/>
-      <c r="C59" s="90" t="s">
+      <c r="A59" s="72"/>
+      <c r="B59" s="68"/>
+      <c r="C59" s="86" t="s">
         <v>69</v>
       </c>
-      <c r="D59" s="90"/>
-      <c r="E59" s="90"/>
-      <c r="F59" s="90"/>
-      <c r="G59" s="90"/>
+      <c r="D59" s="86"/>
+      <c r="E59" s="86"/>
+      <c r="F59" s="86"/>
+      <c r="G59" s="86"/>
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A60" s="66"/>
-      <c r="B60" s="67"/>
-      <c r="C60" s="90" t="s">
+      <c r="A60" s="72"/>
+      <c r="B60" s="68"/>
+      <c r="C60" s="86" t="s">
         <v>64</v>
       </c>
-      <c r="D60" s="90"/>
-      <c r="E60" s="90"/>
-      <c r="F60" s="90"/>
-      <c r="G60" s="90"/>
+      <c r="D60" s="86"/>
+      <c r="E60" s="86"/>
+      <c r="F60" s="86"/>
+      <c r="G60" s="86"/>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A61" s="66"/>
-      <c r="B61" s="67"/>
-      <c r="C61" s="90" t="s">
+      <c r="A61" s="72"/>
+      <c r="B61" s="68"/>
+      <c r="C61" s="86" t="s">
         <v>71</v>
       </c>
-      <c r="D61" s="90"/>
-      <c r="E61" s="90"/>
-      <c r="F61" s="90"/>
-      <c r="G61" s="90"/>
+      <c r="D61" s="86"/>
+      <c r="E61" s="86"/>
+      <c r="F61" s="86"/>
+      <c r="G61" s="86"/>
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A62" s="66"/>
-      <c r="B62" s="67"/>
-      <c r="C62" s="90" t="s">
+      <c r="A62" s="72"/>
+      <c r="B62" s="68"/>
+      <c r="C62" s="86" t="s">
         <v>72</v>
       </c>
-      <c r="D62" s="90"/>
-      <c r="E62" s="90"/>
-      <c r="F62" s="90"/>
-      <c r="G62" s="90"/>
+      <c r="D62" s="86"/>
+      <c r="E62" s="86"/>
+      <c r="F62" s="86"/>
+      <c r="G62" s="86"/>
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A63" s="66"/>
-      <c r="B63" s="67"/>
-      <c r="C63" s="90" t="s">
+      <c r="A63" s="72"/>
+      <c r="B63" s="68"/>
+      <c r="C63" s="86" t="s">
         <v>73</v>
       </c>
-      <c r="D63" s="90"/>
-      <c r="E63" s="90"/>
-      <c r="F63" s="90"/>
-      <c r="G63" s="90"/>
+      <c r="D63" s="86"/>
+      <c r="E63" s="86"/>
+      <c r="F63" s="86"/>
+      <c r="G63" s="86"/>
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A64" s="66">
+      <c r="A64" s="72">
         <v>46217</v>
       </c>
       <c r="B64" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="C64" s="67" t="s">
+      <c r="C64" s="68" t="s">
         <v>15</v>
       </c>
-      <c r="D64" s="67"/>
-      <c r="E64" s="67"/>
-      <c r="F64" s="67"/>
-      <c r="G64" s="67"/>
+      <c r="D64" s="68"/>
+      <c r="E64" s="68"/>
+      <c r="F64" s="68"/>
+      <c r="G64" s="68"/>
     </row>
     <row r="65" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A65" s="66"/>
-      <c r="B65" s="67" t="s">
-        <v>4</v>
-      </c>
-      <c r="C65" s="67" t="s">
+      <c r="A65" s="72"/>
+      <c r="B65" s="68" t="s">
+        <v>4</v>
+      </c>
+      <c r="C65" s="68" t="s">
         <v>39</v>
       </c>
-      <c r="D65" s="67"/>
-      <c r="E65" s="67"/>
-      <c r="F65" s="67"/>
-      <c r="G65" s="67"/>
+      <c r="D65" s="68"/>
+      <c r="E65" s="68"/>
+      <c r="F65" s="68"/>
+      <c r="G65" s="68"/>
     </row>
     <row r="66" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A66" s="66"/>
-      <c r="B66" s="67"/>
-      <c r="C66" s="67" t="s">
+      <c r="A66" s="72"/>
+      <c r="B66" s="68"/>
+      <c r="C66" s="68" t="s">
         <v>74</v>
       </c>
-      <c r="D66" s="67"/>
-      <c r="E66" s="67"/>
-      <c r="F66" s="67"/>
-      <c r="G66" s="67"/>
+      <c r="D66" s="68"/>
+      <c r="E66" s="68"/>
+      <c r="F66" s="68"/>
+      <c r="G66" s="68"/>
     </row>
     <row r="67" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A67" s="6">
@@ -2350,164 +2353,164 @@
       <c r="B67" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="C67" s="67" t="s">
+      <c r="C67" s="68" t="s">
         <v>75</v>
       </c>
-      <c r="D67" s="67"/>
-      <c r="E67" s="67"/>
-      <c r="F67" s="67"/>
-      <c r="G67" s="67"/>
+      <c r="D67" s="68"/>
+      <c r="E67" s="68"/>
+      <c r="F67" s="68"/>
+      <c r="G67" s="68"/>
     </row>
     <row r="68" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A68" s="66">
+      <c r="A68" s="72">
         <v>46220</v>
       </c>
-      <c r="B68" s="67" t="s">
-        <v>4</v>
-      </c>
-      <c r="C68" s="67" t="s">
+      <c r="B68" s="68" t="s">
+        <v>4</v>
+      </c>
+      <c r="C68" s="68" t="s">
         <v>76</v>
       </c>
-      <c r="D68" s="67"/>
-      <c r="E68" s="67"/>
-      <c r="F68" s="67"/>
-      <c r="G68" s="67"/>
+      <c r="D68" s="68"/>
+      <c r="E68" s="68"/>
+      <c r="F68" s="68"/>
+      <c r="G68" s="68"/>
     </row>
     <row r="69" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A69" s="66"/>
-      <c r="B69" s="67"/>
-      <c r="C69" s="67" t="s">
+      <c r="A69" s="72"/>
+      <c r="B69" s="68"/>
+      <c r="C69" s="68" t="s">
         <v>77</v>
       </c>
-      <c r="D69" s="67"/>
-      <c r="E69" s="67"/>
-      <c r="F69" s="67"/>
-      <c r="G69" s="67"/>
+      <c r="D69" s="68"/>
+      <c r="E69" s="68"/>
+      <c r="F69" s="68"/>
+      <c r="G69" s="68"/>
     </row>
     <row r="70" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A70" s="66">
+      <c r="A70" s="72">
         <v>46223</v>
       </c>
-      <c r="B70" s="67" t="s">
-        <v>4</v>
-      </c>
-      <c r="C70" s="68" t="s">
+      <c r="B70" s="68" t="s">
+        <v>4</v>
+      </c>
+      <c r="C70" s="73" t="s">
         <v>78</v>
       </c>
-      <c r="D70" s="69"/>
-      <c r="E70" s="69"/>
-      <c r="F70" s="69"/>
-      <c r="G70" s="70"/>
+      <c r="D70" s="74"/>
+      <c r="E70" s="74"/>
+      <c r="F70" s="74"/>
+      <c r="G70" s="75"/>
     </row>
     <row r="71" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A71" s="66"/>
-      <c r="B71" s="67"/>
-      <c r="C71" s="68" t="s">
+      <c r="A71" s="72"/>
+      <c r="B71" s="68"/>
+      <c r="C71" s="73" t="s">
         <v>79</v>
       </c>
-      <c r="D71" s="69"/>
-      <c r="E71" s="69"/>
-      <c r="F71" s="69"/>
-      <c r="G71" s="70"/>
+      <c r="D71" s="74"/>
+      <c r="E71" s="74"/>
+      <c r="F71" s="74"/>
+      <c r="G71" s="75"/>
     </row>
     <row r="72" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A72" s="66"/>
-      <c r="B72" s="67"/>
-      <c r="C72" s="68" t="s">
+      <c r="A72" s="72"/>
+      <c r="B72" s="68"/>
+      <c r="C72" s="73" t="s">
         <v>80</v>
       </c>
-      <c r="D72" s="69"/>
-      <c r="E72" s="69"/>
-      <c r="F72" s="69"/>
-      <c r="G72" s="70"/>
+      <c r="D72" s="74"/>
+      <c r="E72" s="74"/>
+      <c r="F72" s="74"/>
+      <c r="G72" s="75"/>
     </row>
     <row r="73" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A73" s="66"/>
-      <c r="B73" s="67"/>
-      <c r="C73" s="68" t="s">
+      <c r="A73" s="72"/>
+      <c r="B73" s="68"/>
+      <c r="C73" s="73" t="s">
         <v>81</v>
       </c>
-      <c r="D73" s="69"/>
-      <c r="E73" s="69"/>
-      <c r="F73" s="69"/>
-      <c r="G73" s="70"/>
+      <c r="D73" s="74"/>
+      <c r="E73" s="74"/>
+      <c r="F73" s="74"/>
+      <c r="G73" s="75"/>
     </row>
     <row r="74" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A74" s="66"/>
-      <c r="B74" s="67"/>
-      <c r="C74" s="68" t="s">
+      <c r="A74" s="72"/>
+      <c r="B74" s="68"/>
+      <c r="C74" s="73" t="s">
         <v>39</v>
       </c>
-      <c r="D74" s="69"/>
-      <c r="E74" s="69"/>
-      <c r="F74" s="69"/>
-      <c r="G74" s="70"/>
+      <c r="D74" s="74"/>
+      <c r="E74" s="74"/>
+      <c r="F74" s="74"/>
+      <c r="G74" s="75"/>
     </row>
     <row r="75" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A75" s="66"/>
-      <c r="B75" s="67"/>
-      <c r="C75" s="68" t="s">
+      <c r="A75" s="72"/>
+      <c r="B75" s="68"/>
+      <c r="C75" s="73" t="s">
         <v>82</v>
       </c>
-      <c r="D75" s="69"/>
-      <c r="E75" s="69"/>
-      <c r="F75" s="69"/>
-      <c r="G75" s="70"/>
+      <c r="D75" s="74"/>
+      <c r="E75" s="74"/>
+      <c r="F75" s="74"/>
+      <c r="G75" s="75"/>
     </row>
     <row r="76" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A76" s="66"/>
-      <c r="B76" s="67"/>
-      <c r="C76" s="68" t="s">
+      <c r="A76" s="72"/>
+      <c r="B76" s="68"/>
+      <c r="C76" s="73" t="s">
         <v>72</v>
       </c>
-      <c r="D76" s="69"/>
-      <c r="E76" s="69"/>
-      <c r="F76" s="69"/>
-      <c r="G76" s="70"/>
+      <c r="D76" s="74"/>
+      <c r="E76" s="74"/>
+      <c r="F76" s="74"/>
+      <c r="G76" s="75"/>
     </row>
     <row r="77" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A77" s="66"/>
-      <c r="B77" s="67"/>
-      <c r="C77" s="63" t="s">
+      <c r="A77" s="72"/>
+      <c r="B77" s="68"/>
+      <c r="C77" s="69" t="s">
         <v>83</v>
       </c>
-      <c r="D77" s="64"/>
-      <c r="E77" s="64"/>
-      <c r="F77" s="64"/>
-      <c r="G77" s="65"/>
+      <c r="D77" s="70"/>
+      <c r="E77" s="70"/>
+      <c r="F77" s="70"/>
+      <c r="G77" s="71"/>
     </row>
     <row r="78" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A78" s="66"/>
-      <c r="B78" s="67"/>
-      <c r="C78" s="63" t="s">
+      <c r="A78" s="72"/>
+      <c r="B78" s="68"/>
+      <c r="C78" s="69" t="s">
         <v>84</v>
       </c>
-      <c r="D78" s="64"/>
-      <c r="E78" s="64"/>
-      <c r="F78" s="64"/>
-      <c r="G78" s="65"/>
+      <c r="D78" s="70"/>
+      <c r="E78" s="70"/>
+      <c r="F78" s="70"/>
+      <c r="G78" s="71"/>
     </row>
     <row r="79" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A79" s="66"/>
-      <c r="B79" s="67"/>
-      <c r="C79" s="63" t="s">
+      <c r="A79" s="72"/>
+      <c r="B79" s="68"/>
+      <c r="C79" s="69" t="s">
         <v>85</v>
       </c>
-      <c r="D79" s="64"/>
-      <c r="E79" s="64"/>
-      <c r="F79" s="64"/>
-      <c r="G79" s="65"/>
+      <c r="D79" s="70"/>
+      <c r="E79" s="70"/>
+      <c r="F79" s="70"/>
+      <c r="G79" s="71"/>
     </row>
     <row r="80" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A80" s="66"/>
-      <c r="B80" s="67"/>
-      <c r="C80" s="63" t="s">
+      <c r="A80" s="72"/>
+      <c r="B80" s="68"/>
+      <c r="C80" s="69" t="s">
         <v>86</v>
       </c>
-      <c r="D80" s="64"/>
-      <c r="E80" s="64"/>
-      <c r="F80" s="64"/>
-      <c r="G80" s="65"/>
+      <c r="D80" s="70"/>
+      <c r="E80" s="70"/>
+      <c r="F80" s="70"/>
+      <c r="G80" s="71"/>
     </row>
     <row r="81" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A81" s="6">
@@ -2516,353 +2519,353 @@
       <c r="B81" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="C81" s="67" t="s">
+      <c r="C81" s="68" t="s">
         <v>87</v>
       </c>
-      <c r="D81" s="67"/>
-      <c r="E81" s="67"/>
-      <c r="F81" s="67"/>
-      <c r="G81" s="67"/>
+      <c r="D81" s="68"/>
+      <c r="E81" s="68"/>
+      <c r="F81" s="68"/>
+      <c r="G81" s="68"/>
     </row>
     <row r="82" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A82" s="66">
+      <c r="A82" s="72">
         <v>46225</v>
       </c>
-      <c r="B82" s="67" t="s">
+      <c r="B82" s="68" t="s">
         <v>5</v>
       </c>
-      <c r="C82" s="67" t="s">
+      <c r="C82" s="68" t="s">
         <v>91</v>
       </c>
-      <c r="D82" s="67"/>
-      <c r="E82" s="67"/>
-      <c r="F82" s="67"/>
-      <c r="G82" s="67"/>
+      <c r="D82" s="68"/>
+      <c r="E82" s="68"/>
+      <c r="F82" s="68"/>
+      <c r="G82" s="68"/>
     </row>
     <row r="83" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A83" s="66"/>
-      <c r="B83" s="67"/>
-      <c r="C83" s="67" t="s">
+      <c r="A83" s="72"/>
+      <c r="B83" s="68"/>
+      <c r="C83" s="68" t="s">
         <v>90</v>
       </c>
-      <c r="D83" s="67"/>
-      <c r="E83" s="67"/>
-      <c r="F83" s="67"/>
-      <c r="G83" s="67"/>
+      <c r="D83" s="68"/>
+      <c r="E83" s="68"/>
+      <c r="F83" s="68"/>
+      <c r="G83" s="68"/>
     </row>
     <row r="84" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A84" s="66"/>
-      <c r="B84" s="67"/>
-      <c r="C84" s="67" t="s">
+      <c r="A84" s="72"/>
+      <c r="B84" s="68"/>
+      <c r="C84" s="68" t="s">
         <v>93</v>
       </c>
-      <c r="D84" s="67"/>
-      <c r="E84" s="67"/>
-      <c r="F84" s="67"/>
-      <c r="G84" s="67"/>
+      <c r="D84" s="68"/>
+      <c r="E84" s="68"/>
+      <c r="F84" s="68"/>
+      <c r="G84" s="68"/>
     </row>
     <row r="85" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A85" s="66"/>
-      <c r="B85" s="67" t="s">
-        <v>4</v>
-      </c>
-      <c r="C85" s="67" t="s">
+      <c r="A85" s="72"/>
+      <c r="B85" s="68" t="s">
+        <v>4</v>
+      </c>
+      <c r="C85" s="68" t="s">
         <v>88</v>
       </c>
-      <c r="D85" s="67"/>
-      <c r="E85" s="67"/>
-      <c r="F85" s="67"/>
-      <c r="G85" s="67"/>
+      <c r="D85" s="68"/>
+      <c r="E85" s="68"/>
+      <c r="F85" s="68"/>
+      <c r="G85" s="68"/>
     </row>
     <row r="86" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A86" s="66"/>
-      <c r="B86" s="67"/>
-      <c r="C86" s="67" t="s">
+      <c r="A86" s="72"/>
+      <c r="B86" s="68"/>
+      <c r="C86" s="68" t="s">
         <v>72</v>
       </c>
-      <c r="D86" s="67"/>
-      <c r="E86" s="67"/>
-      <c r="F86" s="67"/>
-      <c r="G86" s="67"/>
+      <c r="D86" s="68"/>
+      <c r="E86" s="68"/>
+      <c r="F86" s="68"/>
+      <c r="G86" s="68"/>
     </row>
     <row r="87" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A87" s="66"/>
-      <c r="B87" s="67"/>
-      <c r="C87" s="67" t="s">
+      <c r="A87" s="72"/>
+      <c r="B87" s="68"/>
+      <c r="C87" s="68" t="s">
         <v>89</v>
       </c>
-      <c r="D87" s="67"/>
-      <c r="E87" s="67"/>
-      <c r="F87" s="67"/>
-      <c r="G87" s="67"/>
+      <c r="D87" s="68"/>
+      <c r="E87" s="68"/>
+      <c r="F87" s="68"/>
+      <c r="G87" s="68"/>
     </row>
     <row r="88" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A88" s="66"/>
-      <c r="B88" s="67"/>
-      <c r="C88" s="67" t="s">
+      <c r="A88" s="72"/>
+      <c r="B88" s="68"/>
+      <c r="C88" s="68" t="s">
         <v>35</v>
       </c>
-      <c r="D88" s="67"/>
-      <c r="E88" s="67"/>
-      <c r="F88" s="67"/>
-      <c r="G88" s="67"/>
+      <c r="D88" s="68"/>
+      <c r="E88" s="68"/>
+      <c r="F88" s="68"/>
+      <c r="G88" s="68"/>
     </row>
     <row r="89" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A89" s="66"/>
-      <c r="B89" s="67"/>
-      <c r="C89" s="68" t="s">
+      <c r="A89" s="72"/>
+      <c r="B89" s="68"/>
+      <c r="C89" s="73" t="s">
         <v>39</v>
       </c>
-      <c r="D89" s="69"/>
-      <c r="E89" s="69"/>
-      <c r="F89" s="69"/>
-      <c r="G89" s="70"/>
+      <c r="D89" s="74"/>
+      <c r="E89" s="74"/>
+      <c r="F89" s="74"/>
+      <c r="G89" s="75"/>
     </row>
     <row r="90" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A90" s="66"/>
-      <c r="B90" s="67"/>
-      <c r="C90" s="67" t="s">
+      <c r="A90" s="72"/>
+      <c r="B90" s="68"/>
+      <c r="C90" s="68" t="s">
         <v>92</v>
       </c>
-      <c r="D90" s="67"/>
-      <c r="E90" s="67"/>
-      <c r="F90" s="67"/>
-      <c r="G90" s="67"/>
+      <c r="D90" s="68"/>
+      <c r="E90" s="68"/>
+      <c r="F90" s="68"/>
+      <c r="G90" s="68"/>
     </row>
     <row r="91" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A91" s="86">
+      <c r="A91" s="81">
         <v>46227</v>
       </c>
-      <c r="B91" s="76" t="s">
+      <c r="B91" s="79" t="s">
         <v>5</v>
       </c>
-      <c r="C91" s="67" t="s">
+      <c r="C91" s="68" t="s">
         <v>94</v>
       </c>
-      <c r="D91" s="67"/>
-      <c r="E91" s="67"/>
-      <c r="F91" s="67"/>
-      <c r="G91" s="67"/>
+      <c r="D91" s="68"/>
+      <c r="E91" s="68"/>
+      <c r="F91" s="68"/>
+      <c r="G91" s="68"/>
     </row>
     <row r="92" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A92" s="88"/>
-      <c r="B92" s="77"/>
-      <c r="C92" s="68" t="s">
+      <c r="A92" s="82"/>
+      <c r="B92" s="80"/>
+      <c r="C92" s="73" t="s">
         <v>95</v>
       </c>
-      <c r="D92" s="69"/>
-      <c r="E92" s="69"/>
-      <c r="F92" s="69"/>
-      <c r="G92" s="70"/>
+      <c r="D92" s="74"/>
+      <c r="E92" s="74"/>
+      <c r="F92" s="74"/>
+      <c r="G92" s="75"/>
     </row>
     <row r="93" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A93" s="66">
+      <c r="A93" s="72">
         <v>46228</v>
       </c>
-      <c r="B93" s="67" t="s">
-        <v>4</v>
-      </c>
-      <c r="C93" s="67" t="s">
+      <c r="B93" s="68" t="s">
+        <v>4</v>
+      </c>
+      <c r="C93" s="68" t="s">
         <v>96</v>
       </c>
-      <c r="D93" s="67"/>
-      <c r="E93" s="67"/>
-      <c r="F93" s="67"/>
-      <c r="G93" s="67"/>
+      <c r="D93" s="68"/>
+      <c r="E93" s="68"/>
+      <c r="F93" s="68"/>
+      <c r="G93" s="68"/>
     </row>
     <row r="94" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A94" s="66"/>
-      <c r="B94" s="67"/>
-      <c r="C94" s="67" t="s">
+      <c r="A94" s="72"/>
+      <c r="B94" s="68"/>
+      <c r="C94" s="68" t="s">
         <v>97</v>
       </c>
-      <c r="D94" s="67"/>
-      <c r="E94" s="67"/>
-      <c r="F94" s="67"/>
-      <c r="G94" s="67"/>
+      <c r="D94" s="68"/>
+      <c r="E94" s="68"/>
+      <c r="F94" s="68"/>
+      <c r="G94" s="68"/>
     </row>
     <row r="95" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A95" s="66"/>
-      <c r="B95" s="67"/>
-      <c r="C95" s="67" t="s">
+      <c r="A95" s="72"/>
+      <c r="B95" s="68"/>
+      <c r="C95" s="68" t="s">
         <v>98</v>
       </c>
-      <c r="D95" s="67"/>
-      <c r="E95" s="67"/>
-      <c r="F95" s="67"/>
-      <c r="G95" s="67"/>
+      <c r="D95" s="68"/>
+      <c r="E95" s="68"/>
+      <c r="F95" s="68"/>
+      <c r="G95" s="68"/>
     </row>
     <row r="96" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A96" s="66"/>
-      <c r="B96" s="67"/>
-      <c r="C96" s="67" t="s">
+      <c r="A96" s="72"/>
+      <c r="B96" s="68"/>
+      <c r="C96" s="68" t="s">
         <v>99</v>
       </c>
-      <c r="D96" s="67"/>
-      <c r="E96" s="67"/>
-      <c r="F96" s="67"/>
-      <c r="G96" s="67"/>
+      <c r="D96" s="68"/>
+      <c r="E96" s="68"/>
+      <c r="F96" s="68"/>
+      <c r="G96" s="68"/>
     </row>
     <row r="97" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A97" s="66"/>
-      <c r="B97" s="67"/>
-      <c r="C97" s="67" t="s">
+      <c r="A97" s="72"/>
+      <c r="B97" s="68"/>
+      <c r="C97" s="68" t="s">
         <v>100</v>
       </c>
-      <c r="D97" s="67"/>
-      <c r="E97" s="67"/>
-      <c r="F97" s="67"/>
-      <c r="G97" s="67"/>
+      <c r="D97" s="68"/>
+      <c r="E97" s="68"/>
+      <c r="F97" s="68"/>
+      <c r="G97" s="68"/>
     </row>
     <row r="98" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A98" s="66"/>
-      <c r="B98" s="67"/>
-      <c r="C98" s="67" t="s">
+      <c r="A98" s="72"/>
+      <c r="B98" s="68"/>
+      <c r="C98" s="68" t="s">
         <v>101</v>
       </c>
-      <c r="D98" s="67"/>
-      <c r="E98" s="67"/>
-      <c r="F98" s="67"/>
-      <c r="G98" s="67"/>
+      <c r="D98" s="68"/>
+      <c r="E98" s="68"/>
+      <c r="F98" s="68"/>
+      <c r="G98" s="68"/>
     </row>
     <row r="99" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A99" s="66">
+      <c r="A99" s="72">
         <v>46230</v>
       </c>
-      <c r="B99" s="67" t="s">
-        <v>4</v>
-      </c>
-      <c r="C99" s="67" t="s">
+      <c r="B99" s="68" t="s">
+        <v>4</v>
+      </c>
+      <c r="C99" s="68" t="s">
         <v>102</v>
       </c>
-      <c r="D99" s="67"/>
-      <c r="E99" s="67"/>
-      <c r="F99" s="67"/>
-      <c r="G99" s="67"/>
+      <c r="D99" s="68"/>
+      <c r="E99" s="68"/>
+      <c r="F99" s="68"/>
+      <c r="G99" s="68"/>
     </row>
     <row r="100" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A100" s="66"/>
-      <c r="B100" s="67"/>
-      <c r="C100" s="67" t="s">
+      <c r="A100" s="72"/>
+      <c r="B100" s="68"/>
+      <c r="C100" s="68" t="s">
         <v>39</v>
       </c>
-      <c r="D100" s="67"/>
-      <c r="E100" s="67"/>
-      <c r="F100" s="67"/>
-      <c r="G100" s="67"/>
+      <c r="D100" s="68"/>
+      <c r="E100" s="68"/>
+      <c r="F100" s="68"/>
+      <c r="G100" s="68"/>
     </row>
     <row r="101" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A101" s="66">
+      <c r="A101" s="72">
         <v>46231</v>
       </c>
       <c r="B101" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="C101" s="92" t="s">
+      <c r="C101" s="78" t="s">
         <v>104</v>
       </c>
-      <c r="D101" s="92"/>
-      <c r="E101" s="92"/>
-      <c r="F101" s="92"/>
-      <c r="G101" s="92"/>
+      <c r="D101" s="78"/>
+      <c r="E101" s="78"/>
+      <c r="F101" s="78"/>
+      <c r="G101" s="78"/>
     </row>
     <row r="102" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A102" s="66"/>
+      <c r="A102" s="72"/>
       <c r="B102" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="C102" s="92" t="s">
+      <c r="C102" s="78" t="s">
         <v>103</v>
       </c>
-      <c r="D102" s="92"/>
-      <c r="E102" s="92"/>
-      <c r="F102" s="92"/>
-      <c r="G102" s="92"/>
+      <c r="D102" s="78"/>
+      <c r="E102" s="78"/>
+      <c r="F102" s="78"/>
+      <c r="G102" s="78"/>
     </row>
     <row r="103" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A103" s="91" t="s">
+      <c r="A103" s="76" t="s">
         <v>105</v>
       </c>
-      <c r="B103" s="67" t="s">
-        <v>4</v>
-      </c>
-      <c r="C103" s="81" t="s">
+      <c r="B103" s="68" t="s">
+        <v>4</v>
+      </c>
+      <c r="C103" s="77" t="s">
         <v>106</v>
       </c>
-      <c r="D103" s="81"/>
-      <c r="E103" s="81"/>
-      <c r="F103" s="81"/>
-      <c r="G103" s="81"/>
+      <c r="D103" s="77"/>
+      <c r="E103" s="77"/>
+      <c r="F103" s="77"/>
+      <c r="G103" s="77"/>
     </row>
     <row r="104" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A104" s="91"/>
-      <c r="B104" s="67"/>
-      <c r="C104" s="67" t="s">
+      <c r="A104" s="76"/>
+      <c r="B104" s="68"/>
+      <c r="C104" s="68" t="s">
         <v>86</v>
       </c>
-      <c r="D104" s="67"/>
-      <c r="E104" s="67"/>
-      <c r="F104" s="67"/>
-      <c r="G104" s="67"/>
+      <c r="D104" s="68"/>
+      <c r="E104" s="68"/>
+      <c r="F104" s="68"/>
+      <c r="G104" s="68"/>
     </row>
     <row r="105" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A105" s="91"/>
-      <c r="B105" s="67"/>
-      <c r="C105" s="67" t="s">
+      <c r="A105" s="76"/>
+      <c r="B105" s="68"/>
+      <c r="C105" s="68" t="s">
         <v>60</v>
       </c>
-      <c r="D105" s="67"/>
-      <c r="E105" s="67"/>
-      <c r="F105" s="67"/>
-      <c r="G105" s="67"/>
+      <c r="D105" s="68"/>
+      <c r="E105" s="68"/>
+      <c r="F105" s="68"/>
+      <c r="G105" s="68"/>
     </row>
     <row r="106" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A106" s="91"/>
-      <c r="B106" s="67"/>
-      <c r="C106" s="67" t="s">
+      <c r="A106" s="76"/>
+      <c r="B106" s="68"/>
+      <c r="C106" s="68" t="s">
         <v>50</v>
       </c>
-      <c r="D106" s="67"/>
-      <c r="E106" s="67"/>
-      <c r="F106" s="67"/>
-      <c r="G106" s="67"/>
+      <c r="D106" s="68"/>
+      <c r="E106" s="68"/>
+      <c r="F106" s="68"/>
+      <c r="G106" s="68"/>
     </row>
     <row r="107" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A107" s="91"/>
-      <c r="B107" s="67"/>
-      <c r="C107" s="67" t="s">
+      <c r="A107" s="76"/>
+      <c r="B107" s="68"/>
+      <c r="C107" s="68" t="s">
         <v>107</v>
       </c>
-      <c r="D107" s="67"/>
-      <c r="E107" s="67"/>
-      <c r="F107" s="67"/>
-      <c r="G107" s="67"/>
+      <c r="D107" s="68"/>
+      <c r="E107" s="68"/>
+      <c r="F107" s="68"/>
+      <c r="G107" s="68"/>
     </row>
     <row r="108" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A108" s="66">
+      <c r="A108" s="72">
         <v>46234</v>
       </c>
-      <c r="B108" s="67" t="s">
-        <v>4</v>
-      </c>
-      <c r="C108" s="67" t="s">
+      <c r="B108" s="68" t="s">
+        <v>4</v>
+      </c>
+      <c r="C108" s="68" t="s">
         <v>108</v>
       </c>
-      <c r="D108" s="67"/>
-      <c r="E108" s="67"/>
-      <c r="F108" s="67"/>
-      <c r="G108" s="67"/>
+      <c r="D108" s="68"/>
+      <c r="E108" s="68"/>
+      <c r="F108" s="68"/>
+      <c r="G108" s="68"/>
     </row>
     <row r="109" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A109" s="66"/>
-      <c r="B109" s="67"/>
-      <c r="C109" s="67" t="s">
+      <c r="A109" s="72"/>
+      <c r="B109" s="68"/>
+      <c r="C109" s="68" t="s">
         <v>39</v>
       </c>
-      <c r="D109" s="67"/>
-      <c r="E109" s="67"/>
-      <c r="F109" s="67"/>
-      <c r="G109" s="67"/>
+      <c r="D109" s="68"/>
+      <c r="E109" s="68"/>
+      <c r="F109" s="68"/>
+      <c r="G109" s="68"/>
     </row>
     <row r="110" spans="1:7" x14ac:dyDescent="0.25">
       <c r="D110" s="10"/>
@@ -2872,68 +2875,67 @@
     </row>
   </sheetData>
   <mergeCells count="147">
-    <mergeCell ref="A103:A107"/>
-    <mergeCell ref="B103:B107"/>
-    <mergeCell ref="C103:G103"/>
-    <mergeCell ref="C104:G104"/>
-    <mergeCell ref="C105:G105"/>
-    <mergeCell ref="C106:G106"/>
-    <mergeCell ref="C107:G107"/>
-    <mergeCell ref="A99:A100"/>
-    <mergeCell ref="B99:B100"/>
-    <mergeCell ref="C99:G99"/>
-    <mergeCell ref="C100:G100"/>
-    <mergeCell ref="C101:G101"/>
-    <mergeCell ref="C102:G102"/>
-    <mergeCell ref="A101:A102"/>
-    <mergeCell ref="B93:B98"/>
-    <mergeCell ref="A93:A98"/>
-    <mergeCell ref="C93:G93"/>
-    <mergeCell ref="C94:G94"/>
-    <mergeCell ref="C95:G95"/>
-    <mergeCell ref="C96:G96"/>
-    <mergeCell ref="C97:G97"/>
-    <mergeCell ref="C98:G98"/>
-    <mergeCell ref="C91:G91"/>
-    <mergeCell ref="C92:G92"/>
-    <mergeCell ref="B91:B92"/>
-    <mergeCell ref="A91:A92"/>
-    <mergeCell ref="A82:A90"/>
-    <mergeCell ref="B82:B84"/>
-    <mergeCell ref="C89:G89"/>
-    <mergeCell ref="C82:G82"/>
-    <mergeCell ref="C83:G83"/>
-    <mergeCell ref="C84:G84"/>
-    <mergeCell ref="C85:G85"/>
-    <mergeCell ref="C86:G86"/>
-    <mergeCell ref="C87:G87"/>
-    <mergeCell ref="C88:G88"/>
-    <mergeCell ref="C90:G90"/>
-    <mergeCell ref="B85:B90"/>
-    <mergeCell ref="C68:G68"/>
-    <mergeCell ref="C69:G69"/>
-    <mergeCell ref="A68:A69"/>
-    <mergeCell ref="B68:B69"/>
-    <mergeCell ref="A64:A66"/>
-    <mergeCell ref="C65:G65"/>
-    <mergeCell ref="C66:G66"/>
-    <mergeCell ref="B65:B66"/>
-    <mergeCell ref="C67:G67"/>
-    <mergeCell ref="C64:G64"/>
-    <mergeCell ref="C81:G81"/>
-    <mergeCell ref="B70:B80"/>
-    <mergeCell ref="A70:A80"/>
-    <mergeCell ref="C70:G70"/>
-    <mergeCell ref="C71:G71"/>
-    <mergeCell ref="C72:G72"/>
-    <mergeCell ref="C73:G73"/>
-    <mergeCell ref="C74:G74"/>
-    <mergeCell ref="C75:G75"/>
-    <mergeCell ref="C76:G76"/>
-    <mergeCell ref="C77:G77"/>
-    <mergeCell ref="C78:G78"/>
-    <mergeCell ref="C79:G79"/>
-    <mergeCell ref="C80:G80"/>
+    <mergeCell ref="A108:A109"/>
+    <mergeCell ref="B108:B109"/>
+    <mergeCell ref="C108:G108"/>
+    <mergeCell ref="C109:G109"/>
+    <mergeCell ref="C38:G38"/>
+    <mergeCell ref="B38:B44"/>
+    <mergeCell ref="C42:G42"/>
+    <mergeCell ref="C43:G43"/>
+    <mergeCell ref="C21:G21"/>
+    <mergeCell ref="C27:G27"/>
+    <mergeCell ref="C28:G28"/>
+    <mergeCell ref="C34:G34"/>
+    <mergeCell ref="C29:G29"/>
+    <mergeCell ref="C31:G31"/>
+    <mergeCell ref="C32:G32"/>
+    <mergeCell ref="C33:G33"/>
+    <mergeCell ref="B20:B22"/>
+    <mergeCell ref="C30:G30"/>
+    <mergeCell ref="C23:G23"/>
+    <mergeCell ref="C20:G20"/>
+    <mergeCell ref="C25:G25"/>
+    <mergeCell ref="C26:G26"/>
+    <mergeCell ref="C22:G22"/>
+    <mergeCell ref="C40:G40"/>
+    <mergeCell ref="C13:G13"/>
+    <mergeCell ref="C41:G41"/>
+    <mergeCell ref="C15:G15"/>
+    <mergeCell ref="C17:G17"/>
+    <mergeCell ref="C19:G19"/>
+    <mergeCell ref="C16:G16"/>
+    <mergeCell ref="B35:B37"/>
+    <mergeCell ref="C35:G35"/>
+    <mergeCell ref="C36:G36"/>
+    <mergeCell ref="C37:G37"/>
+    <mergeCell ref="B18:B19"/>
+    <mergeCell ref="C18:G18"/>
+    <mergeCell ref="B14:B17"/>
+    <mergeCell ref="C47:G47"/>
+    <mergeCell ref="C48:G48"/>
+    <mergeCell ref="C49:G49"/>
+    <mergeCell ref="C50:G50"/>
+    <mergeCell ref="C51:G51"/>
+    <mergeCell ref="C52:G52"/>
+    <mergeCell ref="C53:G53"/>
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="C2:G2"/>
+    <mergeCell ref="A3:A6"/>
+    <mergeCell ref="C3:G3"/>
+    <mergeCell ref="C4:G4"/>
+    <mergeCell ref="C5:G5"/>
+    <mergeCell ref="B4:B6"/>
+    <mergeCell ref="C6:G6"/>
+    <mergeCell ref="C7:G7"/>
+    <mergeCell ref="A7:A13"/>
+    <mergeCell ref="B7:B9"/>
+    <mergeCell ref="B10:B13"/>
+    <mergeCell ref="C8:G8"/>
+    <mergeCell ref="C9:G9"/>
+    <mergeCell ref="C10:G10"/>
+    <mergeCell ref="C11:G11"/>
+    <mergeCell ref="C12:G12"/>
     <mergeCell ref="A35:A44"/>
     <mergeCell ref="C44:G44"/>
     <mergeCell ref="A14:A19"/>
@@ -2958,67 +2960,68 @@
     <mergeCell ref="C45:G45"/>
     <mergeCell ref="B47:B51"/>
     <mergeCell ref="A47:A51"/>
-    <mergeCell ref="C47:G47"/>
-    <mergeCell ref="C48:G48"/>
-    <mergeCell ref="C49:G49"/>
-    <mergeCell ref="C50:G50"/>
-    <mergeCell ref="C51:G51"/>
-    <mergeCell ref="C52:G52"/>
-    <mergeCell ref="C53:G53"/>
-    <mergeCell ref="A1:G1"/>
-    <mergeCell ref="C2:G2"/>
-    <mergeCell ref="A3:A6"/>
-    <mergeCell ref="C3:G3"/>
-    <mergeCell ref="C4:G4"/>
-    <mergeCell ref="C5:G5"/>
-    <mergeCell ref="B4:B6"/>
-    <mergeCell ref="C6:G6"/>
-    <mergeCell ref="C7:G7"/>
-    <mergeCell ref="A7:A13"/>
-    <mergeCell ref="B7:B9"/>
-    <mergeCell ref="B10:B13"/>
-    <mergeCell ref="C8:G8"/>
-    <mergeCell ref="C9:G9"/>
-    <mergeCell ref="C10:G10"/>
-    <mergeCell ref="C11:G11"/>
-    <mergeCell ref="C12:G12"/>
-    <mergeCell ref="C13:G13"/>
-    <mergeCell ref="C41:G41"/>
-    <mergeCell ref="C15:G15"/>
-    <mergeCell ref="C17:G17"/>
-    <mergeCell ref="C19:G19"/>
-    <mergeCell ref="C16:G16"/>
-    <mergeCell ref="B35:B37"/>
-    <mergeCell ref="C35:G35"/>
-    <mergeCell ref="C36:G36"/>
-    <mergeCell ref="C37:G37"/>
-    <mergeCell ref="B18:B19"/>
-    <mergeCell ref="C18:G18"/>
-    <mergeCell ref="B14:B17"/>
-    <mergeCell ref="A108:A109"/>
-    <mergeCell ref="B108:B109"/>
-    <mergeCell ref="C108:G108"/>
-    <mergeCell ref="C109:G109"/>
-    <mergeCell ref="C38:G38"/>
-    <mergeCell ref="B38:B44"/>
-    <mergeCell ref="C42:G42"/>
-    <mergeCell ref="C43:G43"/>
-    <mergeCell ref="C21:G21"/>
-    <mergeCell ref="C27:G27"/>
-    <mergeCell ref="C28:G28"/>
-    <mergeCell ref="C34:G34"/>
-    <mergeCell ref="C29:G29"/>
-    <mergeCell ref="C31:G31"/>
-    <mergeCell ref="C32:G32"/>
-    <mergeCell ref="C33:G33"/>
-    <mergeCell ref="B20:B22"/>
-    <mergeCell ref="C30:G30"/>
-    <mergeCell ref="C23:G23"/>
-    <mergeCell ref="C20:G20"/>
-    <mergeCell ref="C25:G25"/>
-    <mergeCell ref="C26:G26"/>
-    <mergeCell ref="C22:G22"/>
-    <mergeCell ref="C40:G40"/>
+    <mergeCell ref="C81:G81"/>
+    <mergeCell ref="B70:B80"/>
+    <mergeCell ref="A70:A80"/>
+    <mergeCell ref="C70:G70"/>
+    <mergeCell ref="C71:G71"/>
+    <mergeCell ref="C72:G72"/>
+    <mergeCell ref="C73:G73"/>
+    <mergeCell ref="C74:G74"/>
+    <mergeCell ref="C75:G75"/>
+    <mergeCell ref="C76:G76"/>
+    <mergeCell ref="C77:G77"/>
+    <mergeCell ref="C78:G78"/>
+    <mergeCell ref="C79:G79"/>
+    <mergeCell ref="C80:G80"/>
+    <mergeCell ref="C68:G68"/>
+    <mergeCell ref="C69:G69"/>
+    <mergeCell ref="A68:A69"/>
+    <mergeCell ref="B68:B69"/>
+    <mergeCell ref="A64:A66"/>
+    <mergeCell ref="C65:G65"/>
+    <mergeCell ref="C66:G66"/>
+    <mergeCell ref="B65:B66"/>
+    <mergeCell ref="C67:G67"/>
+    <mergeCell ref="C64:G64"/>
+    <mergeCell ref="A82:A90"/>
+    <mergeCell ref="B82:B84"/>
+    <mergeCell ref="C89:G89"/>
+    <mergeCell ref="C82:G82"/>
+    <mergeCell ref="C83:G83"/>
+    <mergeCell ref="C84:G84"/>
+    <mergeCell ref="C85:G85"/>
+    <mergeCell ref="C86:G86"/>
+    <mergeCell ref="C87:G87"/>
+    <mergeCell ref="C88:G88"/>
+    <mergeCell ref="C90:G90"/>
+    <mergeCell ref="B85:B90"/>
+    <mergeCell ref="B93:B98"/>
+    <mergeCell ref="A93:A98"/>
+    <mergeCell ref="C93:G93"/>
+    <mergeCell ref="C94:G94"/>
+    <mergeCell ref="C95:G95"/>
+    <mergeCell ref="C96:G96"/>
+    <mergeCell ref="C97:G97"/>
+    <mergeCell ref="C98:G98"/>
+    <mergeCell ref="C91:G91"/>
+    <mergeCell ref="C92:G92"/>
+    <mergeCell ref="B91:B92"/>
+    <mergeCell ref="A91:A92"/>
+    <mergeCell ref="A103:A107"/>
+    <mergeCell ref="B103:B107"/>
+    <mergeCell ref="C103:G103"/>
+    <mergeCell ref="C104:G104"/>
+    <mergeCell ref="C105:G105"/>
+    <mergeCell ref="C106:G106"/>
+    <mergeCell ref="C107:G107"/>
+    <mergeCell ref="A99:A100"/>
+    <mergeCell ref="B99:B100"/>
+    <mergeCell ref="C99:G99"/>
+    <mergeCell ref="C100:G100"/>
+    <mergeCell ref="C101:G101"/>
+    <mergeCell ref="C102:G102"/>
+    <mergeCell ref="A101:A102"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -3036,15 +3039,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A1" s="79">
+      <c r="A1" s="88">
         <v>46235</v>
       </c>
-      <c r="B1" s="79"/>
-      <c r="C1" s="79"/>
-      <c r="D1" s="79"/>
-      <c r="E1" s="79"/>
-      <c r="F1" s="79"/>
-      <c r="G1" s="79"/>
+      <c r="B1" s="88"/>
+      <c r="C1" s="88"/>
+      <c r="D1" s="88"/>
+      <c r="E1" s="88"/>
+      <c r="F1" s="88"/>
+      <c r="G1" s="88"/>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
@@ -3977,7 +3980,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{35F794F4-B843-4D59-B697-A1CBEF2779DC}">
-  <dimension ref="A1:G59"/>
+  <dimension ref="A1:G61"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.140625" style="10"/>
@@ -4484,9 +4487,6 @@
       <c r="C47" s="25" t="s">
         <v>150</v>
       </c>
-      <c r="D47" s="94"/>
-      <c r="E47" s="94"/>
-      <c r="F47" s="94"/>
       <c r="G47" s="51"/>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.25">
@@ -4514,9 +4514,6 @@
       <c r="C49" s="25" t="s">
         <v>157</v>
       </c>
-      <c r="D49" s="94"/>
-      <c r="E49" s="94"/>
-      <c r="F49" s="94"/>
       <c r="G49" s="51"/>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.25">
@@ -4524,9 +4521,6 @@
       <c r="C50" s="25" t="s">
         <v>126</v>
       </c>
-      <c r="D50" s="94"/>
-      <c r="E50" s="94"/>
-      <c r="F50" s="94"/>
       <c r="G50" s="51"/>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.25">
@@ -4535,9 +4529,6 @@
       <c r="C51" s="25" t="s">
         <v>119</v>
       </c>
-      <c r="D51" s="94"/>
-      <c r="E51" s="94"/>
-      <c r="F51" s="94"/>
       <c r="G51" s="51"/>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.25">
@@ -4546,9 +4537,6 @@
       <c r="C52" s="25" t="s">
         <v>173</v>
       </c>
-      <c r="D52" s="94"/>
-      <c r="E52" s="94"/>
-      <c r="F52" s="94"/>
       <c r="G52" s="51"/>
     </row>
     <row r="53" spans="1:7" x14ac:dyDescent="0.25">
@@ -4557,9 +4545,6 @@
       <c r="C53" s="25" t="s">
         <v>155</v>
       </c>
-      <c r="D53" s="94"/>
-      <c r="E53" s="94"/>
-      <c r="F53" s="94"/>
       <c r="G53" s="51"/>
     </row>
     <row r="54" spans="1:7" x14ac:dyDescent="0.25">
@@ -4568,9 +4553,6 @@
       <c r="C54" s="25" t="s">
         <v>114</v>
       </c>
-      <c r="D54" s="94"/>
-      <c r="E54" s="94"/>
-      <c r="F54" s="94"/>
       <c r="G54" s="51"/>
     </row>
     <row r="55" spans="1:7" x14ac:dyDescent="0.25">
@@ -4579,9 +4561,6 @@
       <c r="C55" s="25" t="s">
         <v>37</v>
       </c>
-      <c r="D55" s="94"/>
-      <c r="E55" s="94"/>
-      <c r="F55" s="94"/>
       <c r="G55" s="51"/>
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.25">
@@ -4590,9 +4569,6 @@
       <c r="C56" s="25" t="s">
         <v>102</v>
       </c>
-      <c r="D56" s="94"/>
-      <c r="E56" s="94"/>
-      <c r="F56" s="94"/>
       <c r="G56" s="51"/>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.25">
@@ -4601,9 +4577,6 @@
       <c r="C57" s="25" t="s">
         <v>174</v>
       </c>
-      <c r="D57" s="94"/>
-      <c r="E57" s="94"/>
-      <c r="F57" s="94"/>
       <c r="G57" s="51"/>
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.25">
@@ -4612,9 +4585,6 @@
       <c r="C58" s="25" t="s">
         <v>78</v>
       </c>
-      <c r="D58" s="94"/>
-      <c r="E58" s="94"/>
-      <c r="F58" s="94"/>
       <c r="G58" s="51"/>
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.25">
@@ -4627,6 +4597,22 @@
       <c r="E59" s="49"/>
       <c r="F59" s="49"/>
       <c r="G59" s="50"/>
+    </row>
+    <row r="60" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A60" s="94">
+        <v>46289</v>
+      </c>
+      <c r="B60" s="10" t="s">
+        <v>4</v>
+      </c>
+      <c r="C60" s="10" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="61" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C61" s="10" t="s">
+        <v>174</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>